<commit_message>
chore: update BrewLite-Tien-do spreadsheet (after voting)
</commit_message>
<xml_diff>
--- a/BrewLite-Tien-do.xlsx
+++ b/BrewLite-Tien-do.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30430"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="202300"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EC2D211-3495-4941-9D3D-A7090A01CF1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{797286BC-1ECF-4576-B37F-6A2CCA7469C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13152" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="135">
   <si>
     <t>ID</t>
   </si>
@@ -89,9 +89,6 @@
     <t>Nền tảng</t>
   </si>
   <si>
-    <t>Khung đã push lên main theo xác nhận của trưởng nhóm.</t>
-  </si>
-  <si>
     <t>Task 2</t>
   </si>
   <si>
@@ -311,12 +308,6 @@
     <t>Bị chặn</t>
   </si>
   <si>
-    <t>Lưu ý</t>
-  </si>
-  <si>
-    <t>A–E là mảng chờ bình chọn lại; cột Người phụ trách đang để trống, chưa gán theo lựa chọn cũ.</t>
-  </si>
-  <si>
     <t>Thời hạn</t>
   </si>
   <si>
@@ -405,6 +396,48 @@
   </si>
   <si>
     <t>README ban đầu đã có; phân công A–E chờ bình chọn lại.</t>
+  </si>
+  <si>
+    <t>Kha (phối hợp Luân, Hùng)</t>
+  </si>
+  <si>
+    <t>Lượng + Luân + Kiệt</t>
+  </si>
+  <si>
+    <t>Lượng + Hùng</t>
+  </si>
+  <si>
+    <t>Hùng</t>
+  </si>
+  <si>
+    <t>Luân</t>
+  </si>
+  <si>
+    <t>Lượng</t>
+  </si>
+  <si>
+    <t>Triệu</t>
+  </si>
+  <si>
+    <t>Task 1 đã dựng khung và push lên main.</t>
+  </si>
+  <si>
+    <t>Owner cập nhật theo kết quả bình chọn ngày 07/10/2026.</t>
+  </si>
+  <si>
+    <t>Lượng làm UI; Hùng làm API thanh toán; Kha hỗ trợ yêu cầu idempotency Task 10.</t>
+  </si>
+  <si>
+    <t>Lượng làm UI xác nhận/lịch sử; Luân hỗ trợ API GET /orders/me; Kiệt lo Docker Compose, README và demo.</t>
+  </si>
+  <si>
+    <t>Kha phụ trách; phối hợp Luân về đơn/tồn kho và Hùng về thanh toán.</t>
+  </si>
+  <si>
+    <t>A–E đã bình chọn: A Triệu, B Lượng, C Luân, D Hùng, E Kha. F: Kiệt.</t>
+  </si>
+  <si>
+    <t>Phân công</t>
   </si>
 </sst>
 </file>
@@ -859,19 +892,19 @@
         <v>1</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>101</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="76" customHeight="1" x14ac:dyDescent="0.5">
@@ -879,79 +912,79 @@
         <v>13</v>
       </c>
       <c r="B2" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="E2" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="F2" s="3" t="s">
         <v>106</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>108</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="76" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A3" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B3" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="E3" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="F3" s="3" t="s">
         <v>111</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="76" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A4" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B4" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="E4" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="C4" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>118</v>
-      </c>
       <c r="F4" s="3" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="76" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A5" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B5" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="E5" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="F5" s="3" t="s">
         <v>120</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>123</v>
       </c>
     </row>
   </sheetData>
@@ -1031,10 +1064,10 @@
         <v>15</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="G2" s="3" t="s">
         <v>16</v>
@@ -1046,255 +1079,289 @@
       <c r="J2" s="3"/>
       <c r="K2" s="3"/>
       <c r="L2" s="3" t="s">
-        <v>18</v>
+        <v>128</v>
       </c>
     </row>
     <row r="3" spans="1:12" ht="58" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A3" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>13</v>
       </c>
       <c r="C3" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="E3" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="F3" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="G3" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3" t="s">
+      <c r="H3" s="3" t="s">
         <v>23</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>24</v>
       </c>
       <c r="I3" s="3"/>
       <c r="J3" s="3"/>
       <c r="K3" s="3"/>
-      <c r="L3" s="3"/>
+      <c r="L3" s="3" t="s">
+        <v>129</v>
+      </c>
     </row>
     <row r="4" spans="1:12" ht="58" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A4" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>13</v>
       </c>
       <c r="C4" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="E4" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="F4" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="H4" s="3" t="s">
         <v>28</v>
-      </c>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>29</v>
       </c>
       <c r="I4" s="3"/>
       <c r="J4" s="3"/>
       <c r="K4" s="3"/>
-      <c r="L4" s="3"/>
+      <c r="L4" s="3" t="s">
+        <v>129</v>
+      </c>
     </row>
     <row r="5" spans="1:12" ht="58" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A5" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>13</v>
       </c>
       <c r="C5" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D5" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="E5" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="H5" s="3" t="s">
         <v>32</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>33</v>
       </c>
       <c r="I5" s="3"/>
       <c r="J5" s="3"/>
       <c r="K5" s="3"/>
-      <c r="L5" s="3"/>
+      <c r="L5" s="3" t="s">
+        <v>129</v>
+      </c>
     </row>
     <row r="6" spans="1:12" ht="58" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A6" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="C6" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="D6" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="E6" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="F6" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="H6" s="3" t="s">
         <v>38</v>
-      </c>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>39</v>
       </c>
       <c r="I6" s="3"/>
       <c r="J6" s="3"/>
       <c r="K6" s="3"/>
-      <c r="L6" s="3"/>
+      <c r="L6" s="3" t="s">
+        <v>129</v>
+      </c>
     </row>
     <row r="7" spans="1:12" ht="58" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A7" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C7" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="B7" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="C7" s="3" t="s">
+      <c r="D7" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="E7" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="H7" s="3" t="s">
         <v>42</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="H7" s="3" t="s">
-        <v>43</v>
       </c>
       <c r="I7" s="3"/>
       <c r="J7" s="3"/>
       <c r="K7" s="3"/>
-      <c r="L7" s="3"/>
+      <c r="L7" s="3" t="s">
+        <v>129</v>
+      </c>
     </row>
     <row r="8" spans="1:12" ht="58" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A8" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C8" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="B8" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="C8" s="3" t="s">
+      <c r="D8" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="E8" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="F8" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="H8" s="3" t="s">
         <v>47</v>
-      </c>
-      <c r="F8" s="3"/>
-      <c r="G8" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="H8" s="3" t="s">
-        <v>48</v>
       </c>
       <c r="I8" s="3"/>
       <c r="J8" s="3"/>
       <c r="K8" s="3"/>
-      <c r="L8" s="3"/>
+      <c r="L8" s="3" t="s">
+        <v>130</v>
+      </c>
     </row>
     <row r="9" spans="1:12" ht="58" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A9" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="C9" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="D9" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="E9" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="F9" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="H9" s="3" t="s">
         <v>53</v>
-      </c>
-      <c r="F9" s="3"/>
-      <c r="G9" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="H9" s="3" t="s">
-        <v>54</v>
       </c>
       <c r="I9" s="3"/>
       <c r="J9" s="3"/>
       <c r="K9" s="3"/>
-      <c r="L9" s="3"/>
+      <c r="L9" s="3" t="s">
+        <v>131</v>
+      </c>
     </row>
     <row r="10" spans="1:12" ht="58" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A10" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C10" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="B10" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="C10" s="3" t="s">
+      <c r="D10" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="E10" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="E10" s="3" t="s">
+      <c r="F10" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="H10" s="3" t="s">
         <v>58</v>
-      </c>
-      <c r="F10" s="3"/>
-      <c r="G10" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="H10" s="3" t="s">
-        <v>59</v>
       </c>
       <c r="I10" s="3"/>
       <c r="J10" s="3"/>
       <c r="K10" s="3"/>
-      <c r="L10" s="3"/>
+      <c r="L10" s="3" t="s">
+        <v>132</v>
+      </c>
     </row>
     <row r="11" spans="1:12" ht="58" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A11" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C11" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="B11" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="C11" s="3" t="s">
+      <c r="D11" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="E11" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="E11" s="3" t="s">
+      <c r="F11" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="H11" s="3" t="s">
         <v>63</v>
-      </c>
-      <c r="F11" s="3"/>
-      <c r="G11" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="H11" s="3" t="s">
-        <v>64</v>
       </c>
       <c r="I11" s="3"/>
       <c r="J11" s="3"/>
@@ -1303,28 +1370,28 @@
     </row>
     <row r="12" spans="1:12" ht="58" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A12" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B12" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="C12" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="D12" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="D12" s="3" t="s">
-        <v>68</v>
-      </c>
       <c r="E12" s="3" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="I12" s="3"/>
       <c r="J12" s="3"/>
@@ -1333,28 +1400,28 @@
     </row>
     <row r="13" spans="1:12" ht="58" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A13" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C13" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="B13" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="C13" s="3" t="s">
+      <c r="D13" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="E13" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="H13" s="3" t="s">
         <v>71</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="G13" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="H13" s="3" t="s">
-        <v>72</v>
       </c>
       <c r="I13" s="3"/>
       <c r="J13" s="3"/>
@@ -1363,60 +1430,60 @@
     </row>
     <row r="14" spans="1:12" ht="58" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A14" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="C14" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="B14" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="C14" s="3" t="s">
+      <c r="D14" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="E14" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="G14" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="E14" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="F14" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="G14" s="3" t="s">
+      <c r="H14" s="3" t="s">
         <v>76</v>
-      </c>
-      <c r="H14" s="3" t="s">
-        <v>77</v>
       </c>
       <c r="I14" s="3"/>
       <c r="J14" s="3"/>
       <c r="K14" s="3"/>
       <c r="L14" s="3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="15" spans="1:12" ht="58" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A15" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C15" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="B15" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="C15" s="3" t="s">
+      <c r="D15" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="D15" s="3" t="s">
+      <c r="E15" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="G15" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="H15" s="3" t="s">
         <v>81</v>
-      </c>
-      <c r="E15" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="F15" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="G15" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="H15" s="3" t="s">
-        <v>82</v>
       </c>
       <c r="I15" s="3"/>
       <c r="J15" s="3"/>
@@ -1448,7 +1515,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="34" customHeight="1" x14ac:dyDescent="0.9">
       <c r="A1" s="9" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
@@ -1457,10 +1524,10 @@
     </row>
     <row r="2" spans="1:6" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A2" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="B2" s="10" t="s">
         <v>84</v>
-      </c>
-      <c r="B2" s="10" t="s">
-        <v>85</v>
       </c>
       <c r="C2" s="8"/>
       <c r="D2" s="8"/>
@@ -1468,10 +1535,10 @@
     </row>
     <row r="3" spans="1:6" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A3" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="B3" s="7" t="s">
         <v>86</v>
-      </c>
-      <c r="B3" s="7" t="s">
-        <v>87</v>
       </c>
       <c r="C3" s="8"/>
       <c r="D3" s="8"/>
@@ -1479,7 +1546,7 @@
     </row>
     <row r="4" spans="1:6" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A4" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B4" s="5" t="str">
         <f>COUNTIF(Backlog!G2:G11,"Đã xong")&amp;" / 10"</f>
@@ -1488,7 +1555,7 @@
     </row>
     <row r="5" spans="1:6" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A5" s="4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B5" s="6">
         <f>COUNTIF(Backlog!G2:G11,"Đã xong")/10</f>
@@ -1497,7 +1564,7 @@
     </row>
     <row r="6" spans="1:6" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A6" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B6" s="5">
         <f>COUNTIF(Backlog!G2:G11,"Chưa bắt đầu")</f>
@@ -1506,7 +1573,7 @@
     </row>
     <row r="7" spans="1:6" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A7" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B7" s="5">
         <f>COUNTIF(Backlog!G2:G11,"Đang làm")</f>
@@ -1515,7 +1582,7 @@
     </row>
     <row r="8" spans="1:6" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A8" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B8" s="5">
         <f>COUNTIF(Backlog!G2:G11,"Chờ review")+COUNTIF(Backlog!G2:G11,"Chờ phối hợp")</f>
@@ -1524,7 +1591,7 @@
     </row>
     <row r="9" spans="1:6" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A9" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B9" s="5">
         <f>COUNTIF(Backlog!G2:G11,"Bị chặn")</f>
@@ -1533,10 +1600,10 @@
     </row>
     <row r="10" spans="1:6" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A10" s="4" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C10" s="8"/>
       <c r="D10" s="8"/>
@@ -1544,10 +1611,10 @@
     </row>
     <row r="11" spans="1:6" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A11" s="4" t="s">
-        <v>92</v>
+        <v>134</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>93</v>
+        <v>133</v>
       </c>
       <c r="C11" s="8"/>
       <c r="D11" s="8"/>
@@ -1555,10 +1622,10 @@
     </row>
     <row r="12" spans="1:6" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A12" s="4" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C12" s="8"/>
       <c r="D12" s="8"/>
@@ -1566,7 +1633,7 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.5">
       <c r="F15" s="1" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: update BrewLite-Tien-do.xlsx with new data
</commit_message>
<xml_diff>
--- a/BrewLite-Tien-do.xlsx
+++ b/BrewLite-Tien-do.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30430"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="202300"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{797286BC-1ECF-4576-B37F-6A2CCA7469C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43EBBB9C-6971-4AB7-8CCE-B33724854A20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13152" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,14 +33,95 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="139">
+  <si>
+    <t>Sprint</t>
+  </si>
+  <si>
+    <t>Mục tiêu</t>
+  </si>
+  <si>
+    <t>Task dự kiến</t>
+  </si>
+  <si>
+    <t>Review: demo gì?</t>
+  </si>
+  <si>
+    <t>Retrospective: câu hỏi</t>
+  </si>
+  <si>
+    <t>Trạng thái tổng quan</t>
+  </si>
+  <si>
+    <t>Sprint 1</t>
+  </si>
+  <si>
+    <t>Dựng nền và hiển thị/chọn món</t>
+  </si>
+  <si>
+    <t>Task 1–4</t>
+  </si>
+  <si>
+    <t>Mở menu; xem chi tiết; chọn size/topping; kiểm tra giá.</t>
+  </si>
+  <si>
+    <t>Điều gì giúp hoàn tất menu? Dữ liệu/API có thống nhất sớm không?</t>
+  </si>
+  <si>
+    <t>Sprint 2</t>
+  </si>
+  <si>
+    <t>Giỏ hàng, tạo đơn và đăng nhập</t>
+  </si>
+  <si>
+    <t>Task 5–7</t>
+  </si>
+  <si>
+    <t>Thêm món vào giỏ; đổi số lượng; tạo đơn; đăng nhập.</t>
+  </si>
+  <si>
+    <t>Có bị chờ API hay thiếu dữ liệu test không? Cần chốt gì trước Sprint 3?</t>
+  </si>
+  <si>
+    <t>Chưa bắt đầu.</t>
+  </si>
+  <si>
+    <t>Sprint 3</t>
+  </si>
+  <si>
+    <t>Thanh toán, nghiệp vụ nâng cao và bàn giao</t>
+  </si>
+  <si>
+    <t>Task 8–10, F-02, F-04</t>
+  </si>
+  <si>
+    <t>Chạy luồng end-to-end; demo thanh toán mock và xác nhận đơn; trình bày Docker Compose.</t>
+  </si>
+  <si>
+    <t>Một điều làm tốt; một vướng mắc; một cải thiện có người theo dõi.</t>
+  </si>
+  <si>
+    <t>Xuyên suốt</t>
+  </si>
+  <si>
+    <t>Điều phối và tài liệu</t>
+  </si>
+  <si>
+    <t>F-01, F-03</t>
+  </si>
+  <si>
+    <t>Kiểm tra README theo từng mốc.</t>
+  </si>
+  <si>
+    <t>Cập nhật khi cần; chốt hành động cụ thể, người theo dõi và hạn kiểm tra.</t>
+  </si>
+  <si>
+    <t>README ban đầu đã có; phân công A–E chờ bình chọn lại.</t>
+  </si>
   <si>
     <t>ID</t>
   </si>
   <si>
-    <t>Sprint</t>
-  </si>
-  <si>
     <t>Task / công việc</t>
   </si>
   <si>
@@ -74,21 +155,27 @@
     <t>Task 1</t>
   </si>
   <si>
-    <t>Sprint 1</t>
-  </si>
-  <si>
     <t>Khởi tạo dự án và cấu trúc</t>
   </si>
   <si>
     <t>[x] Có frontend Next.js và backend NestJS; [x] README, Git, .env.example; [x] build được.</t>
   </si>
   <si>
+    <t>F — Kiệt</t>
+  </si>
+  <si>
+    <t>Kiệt</t>
+  </si>
+  <si>
     <t>Đã xong</t>
   </si>
   <si>
     <t>Nền tảng</t>
   </si>
   <si>
+    <t>Task 1 đã dựng khung và push lên main.</t>
+  </si>
+  <si>
     <t>Task 2</t>
   </si>
   <si>
@@ -101,45 +188,48 @@
     <t>C</t>
   </si>
   <si>
+    <t>Luân</t>
+  </si>
+  <si>
+    <t>Đang làm</t>
+  </si>
+  <si>
+    <t>Sau Task 1; phối hợp A về cấu trúc dữ liệu</t>
+  </si>
+  <si>
+    <t>Owner cập nhật theo kết quả bình chọn ngày 07/10/2026.</t>
+  </si>
+  <si>
+    <t>Task 3</t>
+  </si>
+  <si>
+    <t>Trang menu (frontend)</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>Triệu</t>
+  </si>
+  <si>
+    <t>Sau thống nhất hợp đồng dữ liệu với C; có thể dùng dữ liệu mẫu trước</t>
+  </si>
+  <si>
+    <t>Task 4</t>
+  </si>
+  <si>
+    <t>Chi tiết và tùy chọn sản phẩm</t>
+  </si>
+  <si>
     <t>Chưa bắt đầu</t>
   </si>
   <si>
-    <t>Sau Task 1; phối hợp A về cấu trúc dữ liệu</t>
-  </si>
-  <si>
-    <t>Task 3</t>
-  </si>
-  <si>
-    <t>Trang menu (frontend)</t>
-  </si>
-  <si>
-    <t>[ ] Gọi GET /products; [ ] hiển thị lưới sản phẩm; [ ] có loading/empty state.</t>
-  </si>
-  <si>
-    <t>A</t>
-  </si>
-  <si>
-    <t>Sau thống nhất hợp đồng dữ liệu với C; có thể dùng dữ liệu mẫu trước</t>
-  </si>
-  <si>
-    <t>Task 4</t>
-  </si>
-  <si>
-    <t>Chi tiết và tùy chọn sản phẩm</t>
-  </si>
-  <si>
-    <t>[ ] Trang chi tiết; [ ] chọn size S/M/L và topping; [ ] tính giá theo tùy chọn.</t>
-  </si>
-  <si>
     <t>Dựa trên danh sách sản phẩm Task 2–3</t>
   </si>
   <si>
     <t>Task 5</t>
   </si>
   <si>
-    <t>Sprint 2</t>
-  </si>
-  <si>
     <t>Giỏ hàng (Cart)</t>
   </si>
   <si>
@@ -149,6 +239,9 @@
     <t>B</t>
   </si>
   <si>
+    <t>Lượng</t>
+  </si>
+  <si>
     <t>Phối hợp A để nhận lựa chọn size/topping</t>
   </si>
   <si>
@@ -176,15 +269,18 @@
     <t>D</t>
   </si>
   <si>
+    <t>Hùng</t>
+  </si>
+  <si>
     <t>Phối hợp C về userId trong đơn hàng</t>
   </si>
   <si>
+    <t>Lượng làm UI; Hùng làm API thanh toán; Kha hỗ trợ yêu cầu idempotency Task 10.</t>
+  </si>
+  <si>
     <t>Task 8</t>
   </si>
   <si>
-    <t>Sprint 3</t>
-  </si>
-  <si>
     <t>Thanh toán không tiền mặt (mock)</t>
   </si>
   <si>
@@ -194,9 +290,15 @@
     <t>B + D</t>
   </si>
   <si>
+    <t>Lượng + Hùng</t>
+  </si>
+  <si>
     <t>B làm UI, D làm API; E hỗ trợ idempotency Task 10</t>
   </si>
   <si>
+    <t>Lượng làm UI xác nhận/lịch sử; Luân hỗ trợ API GET /orders/me; Kiệt lo Docker Compose, README và demo.</t>
+  </si>
+  <si>
     <t>Task 9</t>
   </si>
   <si>
@@ -209,9 +311,15 @@
     <t>B + C + F</t>
   </si>
   <si>
+    <t>Lượng + Luân + Kiệt</t>
+  </si>
+  <si>
     <t>B UI; C API; F tích hợp, Compose, README, demo</t>
   </si>
   <si>
+    <t>Kha phụ trách; phối hợp Luân về đơn/tồn kho và Hùng về thanh toán.</t>
+  </si>
+  <si>
     <t>Task 10</t>
   </si>
   <si>
@@ -224,15 +332,15 @@
     <t>E + C + D</t>
   </si>
   <si>
+    <t>Kha (phối hợp Luân, Hùng)</t>
+  </si>
+  <si>
     <t>E phụ trách; C hỗ trợ đơn/tồn kho, D hỗ trợ thanh toán; bắt đầu thiết kế sớm</t>
   </si>
   <si>
     <t>F-01</t>
   </si>
   <si>
-    <t>Xuyên suốt</t>
-  </si>
-  <si>
     <t>Điều phối và thống nhất API</t>
   </si>
   <si>
@@ -260,9 +368,6 @@
     <t>[ ] Yêu cầu cài đặt; [ ] lệnh chạy; [ ] cấu hình .env.example; [ ] hướng dẫn demo và test.</t>
   </si>
   <si>
-    <t>Đang làm</t>
-  </si>
-  <si>
     <t>Cập nhật cùng tiến độ; hoàn thiện ở Sprint 3</t>
   </si>
   <si>
@@ -293,9 +398,6 @@
     <t>Cách dùng</t>
   </si>
   <si>
-    <t>Cập nhật người phụ trách sau khi bình chọn; đổi trạng thái ở sheet Backlog.</t>
-  </si>
-  <si>
     <t>Task chấm điểm hoàn thành</t>
   </si>
   <si>
@@ -308,136 +410,46 @@
     <t>Bị chặn</t>
   </si>
   <si>
+    <t>Kiệt — mảng F</t>
+  </si>
+  <si>
+    <t>Kiệt phụ trách điều phối, tích hợp, README, Docker Compose và demo. Task 1 đã dựng khung và được đánh dấu hoàn thành.</t>
+  </si>
+  <si>
+    <t>Phân công</t>
+  </si>
+  <si>
+    <t>A–E đã bình chọn: A Triệu, B Lượng, C Luân, D Hùng, E Kha. F: Kiệt.</t>
+  </si>
+  <si>
     <t>Thời hạn</t>
   </si>
   <si>
     <t>Chưa có ngày hạn trong thông tin hiện tại; điền khi nhóm xác nhận.</t>
   </si>
   <si>
-    <t>Kiệt</t>
-  </si>
-  <si>
-    <t>Kiệt — mảng F</t>
-  </si>
-  <si>
-    <t>Kiệt phụ trách điều phối, tích hợp, README, Docker Compose và demo. Task 1 đã dựng khung và được đánh dấu hoàn thành.</t>
-  </si>
-  <si>
-    <t>F — Kiệt</t>
-  </si>
-  <si>
-    <t>Mục tiêu</t>
-  </si>
-  <si>
-    <t>Task dự kiến</t>
-  </si>
-  <si>
-    <t>Review: demo gì?</t>
-  </si>
-  <si>
-    <t>Retrospective: câu hỏi</t>
-  </si>
-  <si>
-    <t>Trạng thái tổng quan</t>
-  </si>
-  <si>
-    <t>Dựng nền và hiển thị/chọn món</t>
-  </si>
-  <si>
-    <t>Task 1–4</t>
-  </si>
-  <si>
-    <t>Mở menu; xem chi tiết; chọn size/topping; kiểm tra giá.</t>
-  </si>
-  <si>
-    <t>Điều gì giúp hoàn tất menu? Dữ liệu/API có thống nhất sớm không?</t>
-  </si>
-  <si>
-    <t>Task 1 hoàn tất; Tasks 2–4 chưa bắt đầu.</t>
-  </si>
-  <si>
-    <t>Giỏ hàng, tạo đơn và đăng nhập</t>
-  </si>
-  <si>
-    <t>Task 5–7</t>
-  </si>
-  <si>
-    <t>Thêm món vào giỏ; đổi số lượng; tạo đơn; đăng nhập.</t>
-  </si>
-  <si>
-    <t>Có bị chờ API hay thiếu dữ liệu test không? Cần chốt gì trước Sprint 3?</t>
-  </si>
-  <si>
-    <t>Chưa bắt đầu.</t>
-  </si>
-  <si>
-    <t>Thanh toán, nghiệp vụ nâng cao và bàn giao</t>
-  </si>
-  <si>
-    <t>Task 8–10, F-02, F-04</t>
-  </si>
-  <si>
-    <t>Chạy luồng end-to-end; demo thanh toán mock và xác nhận đơn; trình bày Docker Compose.</t>
-  </si>
-  <si>
-    <t>Một điều làm tốt; một vướng mắc; một cải thiện có người theo dõi.</t>
-  </si>
-  <si>
-    <t>Điều phối và tài liệu</t>
-  </si>
-  <si>
-    <t>F-01, F-03</t>
-  </si>
-  <si>
-    <t>Kiểm tra README theo từng mốc.</t>
-  </si>
-  <si>
-    <t>Cập nhật khi cần; chốt hành động cụ thể, người theo dõi và hạn kiểm tra.</t>
-  </si>
-  <si>
-    <t>README ban đầu đã có; phân công A–E chờ bình chọn lại.</t>
-  </si>
-  <si>
-    <t>Kha (phối hợp Luân, Hùng)</t>
-  </si>
-  <si>
-    <t>Lượng + Luân + Kiệt</t>
-  </si>
-  <si>
-    <t>Lượng + Hùng</t>
-  </si>
-  <si>
-    <t>Hùng</t>
-  </si>
-  <si>
-    <t>Luân</t>
-  </si>
-  <si>
-    <t>Lượng</t>
-  </si>
-  <si>
-    <t>Triệu</t>
-  </si>
-  <si>
-    <t>Task 1 đã dựng khung và push lên main.</t>
-  </si>
-  <si>
-    <t>Owner cập nhật theo kết quả bình chọn ngày 07/10/2026.</t>
-  </si>
-  <si>
-    <t>Lượng làm UI; Hùng làm API thanh toán; Kha hỗ trợ yêu cầu idempotency Task 10.</t>
-  </si>
-  <si>
-    <t>Lượng làm UI xác nhận/lịch sử; Luân hỗ trợ API GET /orders/me; Kiệt lo Docker Compose, README và demo.</t>
-  </si>
-  <si>
-    <t>Kha phụ trách; phối hợp Luân về đơn/tồn kho và Hùng về thanh toán.</t>
-  </si>
-  <si>
-    <t>A–E đã bình chọn: A Triệu, B Lượng, C Luân, D Hùng, E Kha. F: Kiệt.</t>
-  </si>
-  <si>
-    <t>Phân công</t>
+    <t>14/10: Chưa thấy GET /products trong main khi rà soát. Luân xác nhận endpoint đã sẵn sàng chưa, dự kiến hoàn tất và response/schema để phối hợp A.</t>
+  </si>
+  <si>
+    <t>[x] Hiển thị lưới sản phẩm; [x] loading/empty state (đang minh họa bằng dữ liệu mock); [ ] Gọi GET /products khi API sẵn sàng.</t>
+  </si>
+  <si>
+    <t>Giao diện menu đã có và build thành công. Hiện vẫn dùng MOCK_PRODUCTS/loadMockData; cần phối hợp Luân chốt API/response rồi tích hợp, kiểm tra loading/empty với API.</t>
+  </si>
+  <si>
+    <t>[x] Chi tiết sản phẩm; [x] chọn size và topping; [x] tính giá theo tùy chọn (đã thử Americano: 40.000₫ → 45.000₫ size M → 55.000₫ thêm topping).</t>
+  </si>
+  <si>
+    <t>Đã kiểm tra trên giao diện ngày 14/10: giá thay đổi đúng theo size/topping và thêm món vào giỏ. Còn 1 lỗi ESLint ở page.tsx: loadMockData được gọi trong useEffect trước khai báo; nhờ Triệu xử lý rồi kiểm tra lint lại.</t>
+  </si>
+  <si>
+    <t>Kiệt đang điều phối việc chốt API GET /products/response giữa Luân và Triệu, theo dõi tích hợp Task 3 và lỗi lint frontend.</t>
+  </si>
+  <si>
+    <t>Task 1 hoàn tất; Task 2 đang làm; Task 3 đang làm (menu dùng mock, còn tích hợp API); Task 4 chờ review (giá size/topping đã kiểm tra, còn xử lý lint).</t>
+  </si>
+  <si>
+    <t>Cập nhật checklist/trạng thái/ghi chú ở sheet Backlog sau khi xác minh; ghi rõ phụ thuộc và người cần phối hợp.</t>
   </si>
 </sst>
 </file>
@@ -533,12 +545,12 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -889,102 +901,102 @@
   <sheetData>
     <row r="1" spans="1:6" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>97</v>
-      </c>
       <c r="C1" s="2" t="s">
-        <v>98</v>
+        <v>2</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>99</v>
+        <v>3</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>100</v>
+        <v>4</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>101</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="76" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A2" s="3" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>102</v>
+        <v>7</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>103</v>
+        <v>8</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>104</v>
+        <v>9</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>105</v>
+        <v>10</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>106</v>
+        <v>137</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="76" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A3" s="3" t="s">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>107</v>
+        <v>12</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>108</v>
+        <v>13</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>109</v>
+        <v>14</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>110</v>
+        <v>15</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>111</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="76" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A4" s="3" t="s">
-        <v>49</v>
+        <v>17</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>112</v>
+        <v>18</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>113</v>
+        <v>19</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>114</v>
+        <v>20</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>115</v>
+        <v>21</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>111</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="76" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A5" s="3" t="s">
-        <v>65</v>
+        <v>22</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>116</v>
+        <v>23</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>117</v>
+        <v>24</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>118</v>
+        <v>25</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>119</v>
+        <v>26</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>120</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -1014,354 +1026,354 @@
   <sheetData>
     <row r="1" spans="1:12" ht="34" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A1" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>1</v>
-      </c>
       <c r="C1" s="2" t="s">
-        <v>2</v>
+        <v>29</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>3</v>
+        <v>30</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>4</v>
+        <v>31</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>7</v>
+        <v>34</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>8</v>
+        <v>35</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>9</v>
+        <v>36</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>10</v>
+        <v>37</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>11</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="58" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A2" s="3" t="s">
-        <v>12</v>
+        <v>39</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>14</v>
+        <v>40</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>15</v>
+        <v>41</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>96</v>
+        <v>42</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>93</v>
+        <v>43</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>16</v>
+        <v>44</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>17</v>
+        <v>45</v>
       </c>
       <c r="I2" s="3"/>
       <c r="J2" s="3"/>
       <c r="K2" s="3"/>
       <c r="L2" s="3" t="s">
-        <v>128</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3" spans="1:12" ht="58" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A3" s="3" t="s">
-        <v>18</v>
+        <v>47</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>19</v>
+        <v>48</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>20</v>
+        <v>49</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>21</v>
+        <v>50</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>125</v>
+        <v>51</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>22</v>
+        <v>52</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>23</v>
+        <v>53</v>
       </c>
       <c r="I3" s="3"/>
       <c r="J3" s="3"/>
       <c r="K3" s="3"/>
       <c r="L3" s="3" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="4" spans="1:12" ht="58" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A4" s="3" t="s">
-        <v>24</v>
+        <v>55</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>25</v>
+        <v>56</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>26</v>
+        <v>132</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>27</v>
+        <v>57</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>127</v>
+        <v>58</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>22</v>
+        <v>52</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>28</v>
+        <v>59</v>
       </c>
       <c r="I4" s="3"/>
       <c r="J4" s="3"/>
       <c r="K4" s="3"/>
       <c r="L4" s="3" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
     </row>
     <row r="5" spans="1:12" ht="58" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A5" s="3" t="s">
-        <v>29</v>
+        <v>60</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>30</v>
+        <v>61</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>31</v>
+        <v>134</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>27</v>
+        <v>57</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>127</v>
+        <v>58</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>22</v>
+        <v>123</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>32</v>
+        <v>63</v>
       </c>
       <c r="I5" s="3"/>
       <c r="J5" s="3"/>
       <c r="K5" s="3"/>
       <c r="L5" s="3" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="58" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A6" s="3" t="s">
-        <v>33</v>
+        <v>64</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>35</v>
+        <v>65</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>36</v>
+        <v>66</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>37</v>
+        <v>67</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>126</v>
+        <v>68</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>22</v>
+        <v>62</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>38</v>
+        <v>69</v>
       </c>
       <c r="I6" s="3"/>
       <c r="J6" s="3"/>
       <c r="K6" s="3"/>
       <c r="L6" s="3" t="s">
-        <v>129</v>
+        <v>54</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="58" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A7" s="3" t="s">
-        <v>39</v>
+        <v>70</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>40</v>
+        <v>71</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>41</v>
+        <v>72</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>21</v>
+        <v>50</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>125</v>
+        <v>51</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>22</v>
+        <v>62</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>42</v>
+        <v>73</v>
       </c>
       <c r="I7" s="3"/>
       <c r="J7" s="3"/>
       <c r="K7" s="3"/>
       <c r="L7" s="3" t="s">
-        <v>129</v>
+        <v>54</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="58" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A8" s="3" t="s">
-        <v>43</v>
+        <v>74</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>44</v>
+        <v>75</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>45</v>
+        <v>76</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>46</v>
+        <v>77</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>124</v>
+        <v>78</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>22</v>
+        <v>62</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>47</v>
+        <v>79</v>
       </c>
       <c r="I8" s="3"/>
       <c r="J8" s="3"/>
       <c r="K8" s="3"/>
       <c r="L8" s="3" t="s">
-        <v>130</v>
+        <v>80</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="58" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A9" s="3" t="s">
-        <v>48</v>
+        <v>81</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>49</v>
+        <v>17</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>50</v>
+        <v>82</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>51</v>
+        <v>83</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>52</v>
+        <v>84</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>123</v>
+        <v>85</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>22</v>
+        <v>62</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>53</v>
+        <v>86</v>
       </c>
       <c r="I9" s="3"/>
       <c r="J9" s="3"/>
       <c r="K9" s="3"/>
       <c r="L9" s="3" t="s">
-        <v>131</v>
+        <v>87</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="58" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A10" s="3" t="s">
-        <v>54</v>
+        <v>88</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>49</v>
+        <v>17</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>55</v>
+        <v>89</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>56</v>
+        <v>90</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>57</v>
+        <v>91</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>122</v>
+        <v>92</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>22</v>
+        <v>62</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>58</v>
+        <v>93</v>
       </c>
       <c r="I10" s="3"/>
       <c r="J10" s="3"/>
       <c r="K10" s="3"/>
       <c r="L10" s="3" t="s">
-        <v>132</v>
+        <v>94</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="58" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A11" s="3" t="s">
-        <v>59</v>
+        <v>95</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>49</v>
+        <v>17</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>60</v>
+        <v>96</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>61</v>
+        <v>97</v>
       </c>
       <c r="E11" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="G11" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="F11" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="G11" s="3" t="s">
-        <v>22</v>
-      </c>
       <c r="H11" s="3" t="s">
-        <v>63</v>
+        <v>100</v>
       </c>
       <c r="I11" s="3"/>
       <c r="J11" s="3"/>
@@ -1370,58 +1382,60 @@
     </row>
     <row r="12" spans="1:12" ht="58" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A12" s="3" t="s">
-        <v>64</v>
+        <v>101</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>65</v>
+        <v>22</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>66</v>
+        <v>102</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>67</v>
+        <v>103</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>96</v>
+        <v>42</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>93</v>
+        <v>43</v>
       </c>
       <c r="G12" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="H12" s="3" t="s">
         <v>22</v>
-      </c>
-      <c r="H12" s="3" t="s">
-        <v>65</v>
       </c>
       <c r="I12" s="3"/>
       <c r="J12" s="3"/>
       <c r="K12" s="3"/>
-      <c r="L12" s="3"/>
+      <c r="L12" s="3" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="13" spans="1:12" ht="58" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A13" s="3" t="s">
-        <v>68</v>
+        <v>104</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>49</v>
+        <v>17</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>69</v>
+        <v>105</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>70</v>
+        <v>106</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>96</v>
+        <v>42</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>93</v>
+        <v>43</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>22</v>
+        <v>62</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>71</v>
+        <v>107</v>
       </c>
       <c r="I13" s="3"/>
       <c r="J13" s="3"/>
@@ -1430,60 +1444,60 @@
     </row>
     <row r="14" spans="1:12" ht="58" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A14" s="3" t="s">
-        <v>72</v>
+        <v>108</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>65</v>
+        <v>22</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>73</v>
+        <v>109</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>74</v>
+        <v>110</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>96</v>
+        <v>42</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>93</v>
+        <v>43</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>75</v>
+        <v>52</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>76</v>
+        <v>111</v>
       </c>
       <c r="I14" s="3"/>
       <c r="J14" s="3"/>
       <c r="K14" s="3"/>
       <c r="L14" s="3" t="s">
-        <v>77</v>
+        <v>112</v>
       </c>
     </row>
     <row r="15" spans="1:12" ht="58" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A15" s="3" t="s">
-        <v>78</v>
+        <v>113</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>49</v>
+        <v>17</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>79</v>
+        <v>114</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>80</v>
+        <v>115</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>96</v>
+        <v>42</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>93</v>
+        <v>43</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>22</v>
+        <v>62</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>81</v>
+        <v>116</v>
       </c>
       <c r="I15" s="3"/>
       <c r="J15" s="3"/>
@@ -1514,39 +1528,39 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="34" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A1" s="9" t="s">
-        <v>82</v>
-      </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
+      <c r="A1" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
     </row>
     <row r="2" spans="1:6" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A2" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="B2" s="10" t="s">
-        <v>84</v>
-      </c>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
+        <v>118</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
     </row>
     <row r="3" spans="1:6" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A3" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="B3" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8"/>
-      <c r="E3" s="8"/>
+        <v>120</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>138</v>
+      </c>
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
     </row>
     <row r="4" spans="1:6" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A4" s="4" t="s">
-        <v>87</v>
+        <v>121</v>
       </c>
       <c r="B4" s="5" t="str">
         <f>COUNTIF(Backlog!G2:G11,"Đã xong")&amp;" / 10"</f>
@@ -1555,7 +1569,7 @@
     </row>
     <row r="5" spans="1:6" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A5" s="4" t="s">
-        <v>88</v>
+        <v>122</v>
       </c>
       <c r="B5" s="6">
         <f>COUNTIF(Backlog!G2:G11,"Đã xong")/10</f>
@@ -1564,25 +1578,25 @@
     </row>
     <row r="6" spans="1:6" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A6" s="4" t="s">
-        <v>22</v>
+        <v>62</v>
       </c>
       <c r="B6" s="5">
         <f>COUNTIF(Backlog!G2:G11,"Chưa bắt đầu")</f>
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A7" s="4" t="s">
-        <v>75</v>
+        <v>52</v>
       </c>
       <c r="B7" s="5">
         <f>COUNTIF(Backlog!G2:G11,"Đang làm")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A8" s="4" t="s">
-        <v>89</v>
+        <v>123</v>
       </c>
       <c r="B8" s="5">
         <f>COUNTIF(Backlog!G2:G11,"Chờ review")+COUNTIF(Backlog!G2:G11,"Chờ phối hợp")</f>
@@ -1591,7 +1605,7 @@
     </row>
     <row r="9" spans="1:6" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A9" s="4" t="s">
-        <v>90</v>
+        <v>124</v>
       </c>
       <c r="B9" s="5">
         <f>COUNTIF(Backlog!G2:G11,"Bị chặn")</f>
@@ -1600,40 +1614,40 @@
     </row>
     <row r="10" spans="1:6" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A10" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>95</v>
-      </c>
-      <c r="C10" s="8"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="8"/>
+        <v>125</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="C10" s="9"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="9"/>
     </row>
     <row r="11" spans="1:6" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A11" s="4" t="s">
-        <v>134</v>
-      </c>
-      <c r="B11" s="7" t="s">
-        <v>133</v>
-      </c>
-      <c r="C11" s="8"/>
-      <c r="D11" s="8"/>
-      <c r="E11" s="8"/>
+        <v>127</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>128</v>
+      </c>
+      <c r="C11" s="9"/>
+      <c r="D11" s="9"/>
+      <c r="E11" s="9"/>
     </row>
     <row r="12" spans="1:6" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A12" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="B12" s="7" t="s">
-        <v>92</v>
-      </c>
-      <c r="C12" s="8"/>
-      <c r="D12" s="8"/>
-      <c r="E12" s="8"/>
+        <v>129</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>130</v>
+      </c>
+      <c r="C12" s="9"/>
+      <c r="D12" s="9"/>
+      <c r="E12" s="9"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.5">
       <c r="F15" s="1" t="s">
-        <v>93</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactor: update product fetching and reload functionality, replace img with Image component
</commit_message>
<xml_diff>
--- a/BrewLite-Tien-do.xlsx
+++ b/BrewLite-Tien-do.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30430"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="202300"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43EBBB9C-6971-4AB7-8CCE-B33724854A20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D420460D-CEEC-4DF9-AE5C-365C4D192AD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13152" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="141">
   <si>
     <t>Sprint</t>
   </si>
@@ -428,28 +428,34 @@
     <t>Chưa có ngày hạn trong thông tin hiện tại; điền khi nhóm xác nhận.</t>
   </si>
   <si>
-    <t>14/10: Chưa thấy GET /products trong main khi rà soát. Luân xác nhận endpoint đã sẵn sàng chưa, dự kiến hoàn tất và response/schema để phối hợp A.</t>
-  </si>
-  <si>
-    <t>[x] Hiển thị lưới sản phẩm; [x] loading/empty state (đang minh họa bằng dữ liệu mock); [ ] Gọi GET /products khi API sẵn sàng.</t>
-  </si>
-  <si>
-    <t>Giao diện menu đã có và build thành công. Hiện vẫn dùng MOCK_PRODUCTS/loadMockData; cần phối hợp Luân chốt API/response rồi tích hợp, kiểm tra loading/empty với API.</t>
-  </si>
-  <si>
     <t>[x] Chi tiết sản phẩm; [x] chọn size và topping; [x] tính giá theo tùy chọn (đã thử Americano: 40.000₫ → 45.000₫ size M → 55.000₫ thêm topping).</t>
   </si>
   <si>
-    <t>Đã kiểm tra trên giao diện ngày 14/10: giá thay đổi đúng theo size/topping và thêm món vào giỏ. Còn 1 lỗi ESLint ở page.tsx: loadMockData được gọi trong useEffect trước khai báo; nhờ Triệu xử lý rồi kiểm tra lint lại.</t>
-  </si>
-  <si>
-    <t>Kiệt đang điều phối việc chốt API GET /products/response giữa Luân và Triệu, theo dõi tích hợp Task 3 và lỗi lint frontend.</t>
-  </si>
-  <si>
-    <t>Task 1 hoàn tất; Task 2 đang làm; Task 3 đang làm (menu dùng mock, còn tích hợp API); Task 4 chờ review (giá size/topping đã kiểm tra, còn xử lý lint).</t>
-  </si>
-  <si>
     <t>Cập nhật checklist/trạng thái/ghi chú ở sheet Backlog sau khi xác minh; ghi rõ phụ thuộc và người cần phối hợp.</t>
+  </si>
+  <si>
+    <t>Chờ review</t>
+  </si>
+  <si>
+    <t>17/10: GET /products đã chạy và trả 10 sản phẩm; backend build/lint qua. E2E test còn kỳ vọng 4 món nên thất bại; Luân cập nhật test khớp dữ liệu hiện tại rồi chạy lại.</t>
+  </si>
+  <si>
+    <t>[x] Gọi GET /products; [x] hiển thị lưới sản phẩm; [x] có loading/empty state.</t>
+  </si>
+  <si>
+    <t>17/10: Frontend đã nối API, tải và hiển thị 10 món; frontend lint/build qua. Còn cần chỉnh ánh xạ danh mục/mô tả vì Soda việt quất và Matcha Latte hiện bị nhận là Cà phê; phối hợp Luân nếu cần thêm category/description vào API.</t>
+  </si>
+  <si>
+    <t>17/10/2026</t>
+  </si>
+  <si>
+    <t>17/10: Đã kiểm tra chọn size/topping, giá tăng đúng và thêm vào giỏ; frontend lint và build đều qua sau khi sửa lỗi effect và đổi 2 ảnh sang next/image.</t>
+  </si>
+  <si>
+    <t>17/10: API GET /products đã được Luân triển khai và Triệu đã nối frontend. Kiệt theo dõi test backend còn lỗi kỳ vọng số lượng cũ và việc ánh xạ danh mục trên frontend.</t>
+  </si>
+  <si>
+    <t>Task 1 hoàn tất; Task 2 có API trả 10 món, chờ cập nhật test (đang kỳ vọng 4); Task 3 đã nối API nhưng còn chỉnh phân loại một số món; Task 4 đã kiểm tra size/topping và giá, frontend lint/build qua.</t>
   </si>
 </sst>
 </file>
@@ -545,12 +551,12 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -936,7 +942,7 @@
         <v>10</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="76" customHeight="1" x14ac:dyDescent="0.5">
@@ -1114,7 +1120,7 @@
         <v>51</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>52</v>
+        <v>133</v>
       </c>
       <c r="H3" s="3" t="s">
         <v>53</v>
@@ -1123,7 +1129,7 @@
       <c r="J3" s="3"/>
       <c r="K3" s="3"/>
       <c r="L3" s="3" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
     </row>
     <row r="4" spans="1:12" ht="58" customHeight="1" x14ac:dyDescent="0.5">
@@ -1137,7 +1143,7 @@
         <v>56</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>57</v>
@@ -1155,7 +1161,7 @@
       <c r="J4" s="3"/>
       <c r="K4" s="3"/>
       <c r="L4" s="3" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
     </row>
     <row r="5" spans="1:12" ht="58" customHeight="1" x14ac:dyDescent="0.5">
@@ -1169,7 +1175,7 @@
         <v>61</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>57</v>
@@ -1178,16 +1184,18 @@
         <v>58</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>123</v>
+        <v>44</v>
       </c>
       <c r="H5" s="3" t="s">
         <v>63</v>
       </c>
       <c r="I5" s="3"/>
       <c r="J5" s="3"/>
-      <c r="K5" s="3"/>
+      <c r="K5" s="3" t="s">
+        <v>137</v>
+      </c>
       <c r="L5" s="3" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="58" customHeight="1" x14ac:dyDescent="0.5">
@@ -1409,7 +1417,7 @@
       <c r="J12" s="3"/>
       <c r="K12" s="3"/>
       <c r="L12" s="3" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
     </row>
     <row r="13" spans="1:12" ht="58" customHeight="1" x14ac:dyDescent="0.5">
@@ -1528,35 +1536,35 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="34" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="9" t="s">
         <v>117</v>
       </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
     </row>
     <row r="2" spans="1:6" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A2" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="10" t="s">
         <v>119</v>
       </c>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9"/>
-      <c r="E2" s="9"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
     </row>
     <row r="3" spans="1:6" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A3" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="B3" s="10" t="s">
-        <v>138</v>
-      </c>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="9"/>
+      <c r="B3" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="C3" s="8"/>
+      <c r="D3" s="8"/>
+      <c r="E3" s="8"/>
     </row>
     <row r="4" spans="1:6" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A4" s="4" t="s">
@@ -1564,7 +1572,7 @@
       </c>
       <c r="B4" s="5" t="str">
         <f>COUNTIF(Backlog!G2:G11,"Đã xong")&amp;" / 10"</f>
-        <v>1 / 10</v>
+        <v>2 / 10</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.5">
@@ -1573,7 +1581,7 @@
       </c>
       <c r="B5" s="6">
         <f>COUNTIF(Backlog!G2:G11,"Đã xong")/10</f>
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.5">
@@ -1591,7 +1599,7 @@
       </c>
       <c r="B7" s="5">
         <f>COUNTIF(Backlog!G2:G11,"Đang làm")</f>
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.5">
@@ -1600,7 +1608,7 @@
       </c>
       <c r="B8" s="5">
         <f>COUNTIF(Backlog!G2:G11,"Chờ review")+COUNTIF(Backlog!G2:G11,"Chờ phối hợp")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.5">
@@ -1616,34 +1624,34 @@
       <c r="A10" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="7" t="s">
         <v>126</v>
       </c>
-      <c r="C10" s="9"/>
-      <c r="D10" s="9"/>
-      <c r="E10" s="9"/>
+      <c r="C10" s="8"/>
+      <c r="D10" s="8"/>
+      <c r="E10" s="8"/>
     </row>
     <row r="11" spans="1:6" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A11" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="B11" s="10" t="s">
+      <c r="B11" s="7" t="s">
         <v>128</v>
       </c>
-      <c r="C11" s="9"/>
-      <c r="D11" s="9"/>
-      <c r="E11" s="9"/>
+      <c r="C11" s="8"/>
+      <c r="D11" s="8"/>
+      <c r="E11" s="8"/>
     </row>
     <row r="12" spans="1:6" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A12" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="B12" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="C12" s="9"/>
-      <c r="D12" s="9"/>
-      <c r="E12" s="9"/>
+      <c r="C12" s="8"/>
+      <c r="D12" s="8"/>
+      <c r="E12" s="8"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.5">
       <c r="F15" s="1" t="s">

</xml_diff>

<commit_message>
docs: update README and add API contract documentation
</commit_message>
<xml_diff>
--- a/BrewLite-Tien-do.xlsx
+++ b/BrewLite-Tien-do.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30430"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="202300"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D420460D-CEEC-4DF9-AE5C-365C4D192AD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D32E8EF-B140-4F16-BC70-226375A098F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13152" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="141">
   <si>
     <t>Sprint</t>
   </si>
@@ -371,9 +371,6 @@
     <t>Cập nhật cùng tiến độ; hoàn thiện ở Sprint 3</t>
   </si>
   <si>
-    <t>README ban đầu đã có, tiếp tục bổ sung.</t>
-  </si>
-  <si>
     <t>F-04</t>
   </si>
   <si>
@@ -452,10 +449,13 @@
     <t>17/10: Đã kiểm tra chọn size/topping, giá tăng đúng và thêm vào giỏ; frontend lint và build đều qua sau khi sửa lỗi effect và đổi 2 ảnh sang next/image.</t>
   </si>
   <si>
-    <t>17/10: API GET /products đã được Luân triển khai và Triệu đã nối frontend. Kiệt theo dõi test backend còn lỗi kỳ vọng số lượng cũ và việc ánh xạ danh mục trên frontend.</t>
-  </si>
-  <si>
     <t>Task 1 hoàn tất; Task 2 có API trả 10 món, chờ cập nhật test (đang kỳ vọng 4); Task 3 đã nối API nhưng còn chỉnh phân loại một số món; Task 4 đã kiểm tra size/topping và giá, frontend lint/build qua.</t>
+  </si>
+  <si>
+    <t>17/10: Đã ghi hợp đồng GET /products đã xác minh và danh sách quyết định còn mở tại docs/api-contracts.md. Còn cần Luân/Triệu thống nhất category/description; Luân cập nhật e2e test; Luân/Lượng chốt POST /orders; Luân/Hùng xác nhận liên kết user với đơn.</t>
+  </si>
+  <si>
+    <t>17/10: Đã cập nhật README hướng dẫn cài dependencies, chạy frontend/backend, API hiện có, lệnh kiểm tra và ghi chú rõ e2e test đang lỗi kỳ vọng số lượng cũ.</t>
   </si>
 </sst>
 </file>
@@ -942,7 +942,7 @@
         <v>10</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="76" customHeight="1" x14ac:dyDescent="0.5">
@@ -1120,7 +1120,7 @@
         <v>51</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="H3" s="3" t="s">
         <v>53</v>
@@ -1129,7 +1129,7 @@
       <c r="J3" s="3"/>
       <c r="K3" s="3"/>
       <c r="L3" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="4" spans="1:12" ht="58" customHeight="1" x14ac:dyDescent="0.5">
@@ -1143,7 +1143,7 @@
         <v>56</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>57</v>
@@ -1161,7 +1161,7 @@
       <c r="J4" s="3"/>
       <c r="K4" s="3"/>
       <c r="L4" s="3" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="5" spans="1:12" ht="58" customHeight="1" x14ac:dyDescent="0.5">
@@ -1175,7 +1175,7 @@
         <v>61</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>57</v>
@@ -1192,10 +1192,10 @@
       <c r="I5" s="3"/>
       <c r="J5" s="3"/>
       <c r="K5" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="L5" s="3" t="s">
         <v>137</v>
-      </c>
-      <c r="L5" s="3" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="58" customHeight="1" x14ac:dyDescent="0.5">
@@ -1470,30 +1470,32 @@
         <v>43</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="H14" s="3" t="s">
         <v>111</v>
       </c>
       <c r="I14" s="3"/>
       <c r="J14" s="3"/>
-      <c r="K14" s="3"/>
+      <c r="K14" s="3" t="s">
+        <v>136</v>
+      </c>
       <c r="L14" s="3" t="s">
-        <v>112</v>
+        <v>140</v>
       </c>
     </row>
     <row r="15" spans="1:12" ht="58" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A15" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>17</v>
       </c>
       <c r="C15" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="D15" s="3" t="s">
         <v>114</v>
-      </c>
-      <c r="D15" s="3" t="s">
-        <v>115</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>42</v>
@@ -1505,7 +1507,7 @@
         <v>62</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="I15" s="3"/>
       <c r="J15" s="3"/>
@@ -1537,7 +1539,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="34" customHeight="1" x14ac:dyDescent="0.9">
       <c r="A1" s="9" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
@@ -1546,10 +1548,10 @@
     </row>
     <row r="2" spans="1:6" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A2" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="B2" s="10" t="s">
         <v>118</v>
-      </c>
-      <c r="B2" s="10" t="s">
-        <v>119</v>
       </c>
       <c r="C2" s="8"/>
       <c r="D2" s="8"/>
@@ -1557,10 +1559,10 @@
     </row>
     <row r="3" spans="1:6" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A3" s="4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C3" s="8"/>
       <c r="D3" s="8"/>
@@ -1568,7 +1570,7 @@
     </row>
     <row r="4" spans="1:6" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A4" s="4" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B4" s="5" t="str">
         <f>COUNTIF(Backlog!G2:G11,"Đã xong")&amp;" / 10"</f>
@@ -1577,7 +1579,7 @@
     </row>
     <row r="5" spans="1:6" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A5" s="4" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B5" s="6">
         <f>COUNTIF(Backlog!G2:G11,"Đã xong")/10</f>
@@ -1604,7 +1606,7 @@
     </row>
     <row r="8" spans="1:6" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A8" s="4" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B8" s="5">
         <f>COUNTIF(Backlog!G2:G11,"Chờ review")+COUNTIF(Backlog!G2:G11,"Chờ phối hợp")</f>
@@ -1613,7 +1615,7 @@
     </row>
     <row r="9" spans="1:6" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A9" s="4" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B9" s="5">
         <f>COUNTIF(Backlog!G2:G11,"Bị chặn")</f>
@@ -1622,10 +1624,10 @@
     </row>
     <row r="10" spans="1:6" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A10" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="B10" s="7" t="s">
         <v>125</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>126</v>
       </c>
       <c r="C10" s="8"/>
       <c r="D10" s="8"/>
@@ -1633,10 +1635,10 @@
     </row>
     <row r="11" spans="1:6" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A11" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="B11" s="7" t="s">
         <v>127</v>
-      </c>
-      <c r="B11" s="7" t="s">
-        <v>128</v>
       </c>
       <c r="C11" s="8"/>
       <c r="D11" s="8"/>
@@ -1644,10 +1646,10 @@
     </row>
     <row r="12" spans="1:6" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A12" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="B12" s="7" t="s">
         <v>129</v>
-      </c>
-      <c r="B12" s="7" t="s">
-        <v>130</v>
       </c>
       <c r="C12" s="8"/>
       <c r="D12" s="8"/>

</xml_diff>

<commit_message>
chore: update BrewLite-Tien-do.xlsx with new content
</commit_message>
<xml_diff>
--- a/BrewLite-Tien-do.xlsx
+++ b/BrewLite-Tien-do.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:ns4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:ns5="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:ns7="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ns1:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30430"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="202300"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D32E8EF-B140-4F16-BC70-226375A098F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <ns2:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D32E8EF-B140-4F16-BC70-226375A098F2}" ns3:coauthVersionLast="47" ns3:coauthVersionMax="47" ns4:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13152" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13152" ns5:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sprint" sheetId="3" r:id="rId1"/>
@@ -15,18 +15,18 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase">Sprint!$A$1:$F$5</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1" forceFullCalc="1"/>
   <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
+    <ext uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <ns7:calcFeatures>
+        <ns7:feature name="microsoft.com:RD"/>
+        <ns7:feature name="microsoft.com:Single"/>
+        <ns7:feature name="microsoft.com:FV"/>
+        <ns7:feature name="microsoft.com:CNMTM"/>
+        <ns7:feature name="microsoft.com:LET_WF"/>
+        <ns7:feature name="microsoft.com:LAMBDA_WF"/>
+        <ns7:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </ns7:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -892,9 +892,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F5"/>
-  <sheetFormatPr defaultRowHeight="12.9" customHeight="1" x14ac:dyDescent="0.5"/>
+  <sheetFormatPr defaultRowHeight="12.9" customHeight="1" ns3:dyDescent="0.5"/>
   <cols>
     <col min="1" max="1" width="16.6171875" style="1" customWidth="1"/>
     <col min="2" max="2" width="38.6171875" style="1" customWidth="1"/>
@@ -905,7 +905,7 @@
     <col min="8" max="16384" width="8.76171875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:6" ht="32.049999999999997" customHeight="1" ns3:dyDescent="0.5">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -925,7 +925,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="76" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="2" spans="1:6" ht="76" customHeight="1" ns3:dyDescent="0.5">
       <c r="A2" s="3" t="s">
         <v>6</v>
       </c>
@@ -941,11 +941,13 @@
       <c r="E2" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="3" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" ht="76" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Cập nhật 22/10: Task 1 và 4 hoàn tất; Task 2 đã chuyển GET /products sang PostgreSQL/Prisma, có migration và seed, đang chờ chạy kiểm tra DB/endpoint và cập nhật README; Task 3 đã có menu nối API nhưng cần rà soát phân loại món.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="76" customHeight="1" ns3:dyDescent="0.5">
       <c r="A3" s="3" t="s">
         <v>11</v>
       </c>
@@ -961,11 +963,13 @@
       <c r="E3" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="F3" s="3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" ht="76" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Cập nhật 22/10: Task 5 (giỏ hàng) và Task 6 (API tạo đơn) đã merge PR #9 và #10; Task 7 (đăng ký/đăng nhập JWT) chưa thấy PR trên GitHub.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="76" customHeight="1" ns3:dyDescent="0.5">
       <c r="A4" s="3" t="s">
         <v>17</v>
       </c>
@@ -985,7 +989,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="76" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="5" spans="1:6" ht="76" customHeight="1" ns3:dyDescent="0.5">
       <c r="A5" s="3" t="s">
         <v>22</v>
       </c>
@@ -1011,9 +1015,9 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:L15"/>
-  <sheetFormatPr defaultRowHeight="12.9" customHeight="1" x14ac:dyDescent="0.5"/>
+  <sheetFormatPr defaultRowHeight="12.9" customHeight="1" ns3:dyDescent="0.5"/>
   <cols>
     <col min="1" max="1" width="12.6171875" style="1" customWidth="1"/>
     <col min="2" max="2" width="13.6171875" style="1" customWidth="1"/>
@@ -1030,7 +1034,7 @@
     <col min="14" max="16384" width="8.76171875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="34" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:12" ht="34" customHeight="1" ns3:dyDescent="0.5">
       <c r="A1" s="2" t="s">
         <v>28</v>
       </c>
@@ -1068,7 +1072,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="58" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="2" spans="1:12" ht="58" customHeight="1" ns3:dyDescent="0.5">
       <c r="A2" s="3" t="s">
         <v>39</v>
       </c>
@@ -1100,7 +1104,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="58" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="3" spans="1:12" ht="58" customHeight="1" ns3:dyDescent="0.5">
       <c r="A3" s="3" t="s">
         <v>47</v>
       </c>
@@ -1128,11 +1132,13 @@
       <c r="I3" s="3"/>
       <c r="J3" s="3"/>
       <c r="K3" s="3"/>
-      <c r="L3" s="3" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" ht="58" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>21/10: PR #11 đã merge; GET /products đọc từ PostgreSQL/Prisma. Có migration và seed 10 sản phẩm. Cần kiểm thử migration + seed + endpoint trên môi trường sạch; README hiện vẫn mô tả sản phẩm trong bộ nhớ, cần cập nhật.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" spans="1:12" ht="58" customHeight="1" ns3:dyDescent="0.5">
       <c r="A4" s="3" t="s">
         <v>55</v>
       </c>
@@ -1160,11 +1166,13 @@
       <c r="I4" s="3"/>
       <c r="J4" s="3"/>
       <c r="K4" s="3"/>
-      <c r="L4" s="3" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" ht="58" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>22/10: PR #8 đã merge; menu gọi API và có trạng thái tải/rỗng/lỗi. Frontend hiện suy ra danh mục theo tên; Soda việt quất và Matcha Latte được xếp vào “Khác”. Cần nhóm xác nhận cách phân loại này có đúng mong muốn không.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" spans="1:12" ht="58" customHeight="1" ns3:dyDescent="0.5">
       <c r="A5" s="3" t="s">
         <v>60</v>
       </c>
@@ -1198,7 +1206,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="58" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="6" spans="1:12" ht="58" customHeight="1" ns3:dyDescent="0.5">
       <c r="A6" s="3" t="s">
         <v>64</v>
       </c>
@@ -1217,20 +1225,28 @@
       <c r="F6" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="G6" s="3" t="s">
-        <v>62</v>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>Đã xong</t>
+        </is>
       </c>
       <c r="H6" s="3" t="s">
         <v>69</v>
       </c>
       <c r="I6" s="3"/>
       <c r="J6" s="3"/>
-      <c r="K6" s="3"/>
-      <c r="L6" s="3" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" ht="58" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="K6" s="3" t="inlineStr">
+        <is>
+          <t>20/10/2026</t>
+        </is>
+      </c>
+      <c r="L6" s="3" t="inlineStr">
+        <is>
+          <t>20/10: PR #9 đã merge; giỏ hàng có thêm/sửa/xóa món, tính tổng và lưu localStorage. Cần kiểm tra lại luồng tích hợp sau khi ghép API/database.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" spans="1:12" ht="58" customHeight="1" ns3:dyDescent="0.5">
       <c r="A7" s="3" t="s">
         <v>70</v>
       </c>
@@ -1249,20 +1265,28 @@
       <c r="F7" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="G7" s="3" t="s">
-        <v>62</v>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Đã xong</t>
+        </is>
       </c>
       <c r="H7" s="3" t="s">
         <v>73</v>
       </c>
       <c r="I7" s="3"/>
       <c r="J7" s="3"/>
-      <c r="K7" s="3"/>
-      <c r="L7" s="3" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" ht="58" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="K7" s="3" t="inlineStr">
+        <is>
+          <t>20/10/2026</t>
+        </is>
+      </c>
+      <c r="L7" s="3" t="inlineStr">
+        <is>
+          <t>20/10: PR #10 đã merge; POST /orders validate giỏ, tính giá phía server, trả orderCode và trạng thái PENDING; có e2e tests. Đơn vẫn lưu trong bộ nhớ và mất khi backend khởi động lại; cần xác nhận đây là giới hạn chấp nhận được cho Task 6.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" spans="1:12" ht="58" customHeight="1" ns3:dyDescent="0.5">
       <c r="A8" s="3" t="s">
         <v>74</v>
       </c>
@@ -1294,7 +1318,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="9" spans="1:12" ht="58" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="9" spans="1:12" ht="58" customHeight="1" ns3:dyDescent="0.5">
       <c r="A9" s="3" t="s">
         <v>81</v>
       </c>
@@ -1326,7 +1350,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="10" spans="1:12" ht="58" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="10" spans="1:12" ht="58" customHeight="1" ns3:dyDescent="0.5">
       <c r="A10" s="3" t="s">
         <v>88</v>
       </c>
@@ -1358,7 +1382,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="11" spans="1:12" ht="58" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="11" spans="1:12" ht="58" customHeight="1" ns3:dyDescent="0.5">
       <c r="A11" s="3" t="s">
         <v>95</v>
       </c>
@@ -1388,7 +1412,7 @@
       <c r="K11" s="3"/>
       <c r="L11" s="3"/>
     </row>
-    <row r="12" spans="1:12" ht="58" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="12" spans="1:12" ht="58" customHeight="1" ns3:dyDescent="0.5">
       <c r="A12" s="3" t="s">
         <v>101</v>
       </c>
@@ -1420,7 +1444,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="13" spans="1:12" ht="58" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="13" spans="1:12" ht="58" customHeight="1" ns3:dyDescent="0.5">
       <c r="A13" s="3" t="s">
         <v>104</v>
       </c>
@@ -1450,7 +1474,7 @@
       <c r="K13" s="3"/>
       <c r="L13" s="3"/>
     </row>
-    <row r="14" spans="1:12" ht="58" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="14" spans="1:12" ht="58" customHeight="1" ns3:dyDescent="0.5">
       <c r="A14" s="3" t="s">
         <v>108</v>
       </c>
@@ -1484,7 +1508,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="15" spans="1:12" ht="58" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="15" spans="1:12" ht="58" customHeight="1" ns3:dyDescent="0.5">
       <c r="A15" s="3" t="s">
         <v>112</v>
       </c>
@@ -1515,9 +1539,9 @@
       <c r="L15" s="3"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L15" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <autoFilter ref="A1:L15" ns2:uid="{00000000-0009-0000-0000-000001000000}"/>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G15" xr:uid="{00000000-0002-0000-0100-000000000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G15" ns2:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"Chưa bắt đầu,Đang làm,Chờ phối hợp,Chờ review,Đã xong,Bị chặn"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1526,9 +1550,9 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:F15"/>
-  <sheetFormatPr defaultRowHeight="12.9" customHeight="1" x14ac:dyDescent="0.5"/>
+  <sheetFormatPr defaultRowHeight="12.9" customHeight="1" ns3:dyDescent="0.5"/>
   <cols>
     <col min="1" max="1" width="27.6171875" style="1" customWidth="1"/>
     <col min="2" max="2" width="48.6171875" style="1" customWidth="1"/>
@@ -1537,7 +1561,7 @@
     <col min="7" max="16384" width="8.76171875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="34" customHeight="1" x14ac:dyDescent="0.9">
+    <row r="1" spans="1:6" ht="34" customHeight="1" ns3:dyDescent="0.9">
       <c r="A1" s="9" t="s">
         <v>116</v>
       </c>
@@ -1546,7 +1570,7 @@
       <c r="D1" s="9"/>
       <c r="E1" s="9"/>
     </row>
-    <row r="2" spans="1:6" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="2" spans="1:6" ht="32.049999999999997" customHeight="1" ns3:dyDescent="0.5">
       <c r="A2" s="4" t="s">
         <v>117</v>
       </c>
@@ -1557,7 +1581,7 @@
       <c r="D2" s="8"/>
       <c r="E2" s="8"/>
     </row>
-    <row r="3" spans="1:6" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="3" spans="1:6" ht="32.049999999999997" customHeight="1" ns3:dyDescent="0.5">
       <c r="A3" s="4" t="s">
         <v>119</v>
       </c>
@@ -1568,34 +1592,34 @@
       <c r="D3" s="8"/>
       <c r="E3" s="8"/>
     </row>
-    <row r="4" spans="1:6" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="4" spans="1:6" ht="32.049999999999997" customHeight="1" ns3:dyDescent="0.5">
       <c r="A4" s="4" t="s">
         <v>120</v>
       </c>
       <c r="B4" s="5" t="str">
         <f>COUNTIF(Backlog!G2:G11,"Đã xong")&amp;" / 10"</f>
-        <v>2 / 10</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.5">
+        <v>4 / 10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="32.049999999999997" customHeight="1" ns3:dyDescent="0.5">
       <c r="A5" s="4" t="s">
         <v>121</v>
       </c>
       <c r="B5" s="6">
         <f>COUNTIF(Backlog!G2:G11,"Đã xong")/10</f>
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.5">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="32.049999999999997" customHeight="1" ns3:dyDescent="0.5">
       <c r="A6" s="4" t="s">
         <v>62</v>
       </c>
       <c r="B6" s="5">
         <f>COUNTIF(Backlog!G2:G11,"Chưa bắt đầu")</f>
-        <v>6</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="32.049999999999997" customHeight="1" ns3:dyDescent="0.5">
       <c r="A7" s="4" t="s">
         <v>52</v>
       </c>
@@ -1604,7 +1628,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="8" spans="1:6" ht="32.049999999999997" customHeight="1" ns3:dyDescent="0.5">
       <c r="A8" s="4" t="s">
         <v>122</v>
       </c>
@@ -1613,7 +1637,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="9" spans="1:6" ht="32.049999999999997" customHeight="1" ns3:dyDescent="0.5">
       <c r="A9" s="4" t="s">
         <v>123</v>
       </c>
@@ -1622,7 +1646,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="10" spans="1:6" ht="32.049999999999997" customHeight="1" ns3:dyDescent="0.5">
       <c r="A10" s="4" t="s">
         <v>124</v>
       </c>
@@ -1633,7 +1657,7 @@
       <c r="D10" s="8"/>
       <c r="E10" s="8"/>
     </row>
-    <row r="11" spans="1:6" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="11" spans="1:6" ht="32.049999999999997" customHeight="1" ns3:dyDescent="0.5">
       <c r="A11" s="4" t="s">
         <v>126</v>
       </c>
@@ -1644,7 +1668,7 @@
       <c r="D11" s="8"/>
       <c r="E11" s="8"/>
     </row>
-    <row r="12" spans="1:6" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="12" spans="1:6" ht="32.049999999999997" customHeight="1" ns3:dyDescent="0.5">
       <c r="A12" s="4" t="s">
         <v>128</v>
       </c>
@@ -1655,7 +1679,7 @@
       <c r="D12" s="8"/>
       <c r="E12" s="8"/>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.5">
+    <row r="15" spans="1:6" ns3:dyDescent="0.5">
       <c r="F15" s="1" t="s">
         <v>43</v>
       </c>
@@ -1670,7 +1694,7 @@
     <mergeCell ref="B11:E11"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1" xr:uid="{00000000-0004-0000-0200-000000000000}"/>
+    <hyperlink ref="B2" r:id="rId1" ns2:uid="{00000000-0004-0000-0200-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
ci: add BrewLite validation workflow
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/BrewLite-Tien-do.xlsx
+++ b/BrewLite-Tien-do.xlsx
@@ -943,7 +943,7 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>Cập nhật 22/10: Task 1 và 4 hoàn tất; Task 2 đã chuyển GET /products sang PostgreSQL/Prisma, có migration và seed, đang chờ chạy kiểm tra DB/endpoint và cập nhật README; Task 3 đã có menu nối API nhưng cần rà soát phân loại món.</t>
+          <t>Cập nhật 22/10: Task 1, 4 hoàn tất. Task 2 có PostgreSQL/Prisma + migration/seed, chờ kiểm tra kết nối thật; Task 3 menu đã nối API, cần xác nhận phân loại món.</t>
         </is>
       </c>
     </row>
@@ -965,7 +965,7 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Cập nhật 22/10: Task 5 (giỏ hàng) và Task 6 (API tạo đơn) đã merge PR #9 và #10; Task 7 (đăng ký/đăng nhập JWT) chưa thấy PR trên GitHub.</t>
+          <t>Task 5 và 6 đã merge. Task 7 đang làm trên branch hung, chưa có PR; cần hoàn thiện bảo vệ route đặt đơn và test trước khi chốt Sprint 2.</t>
         </is>
       </c>
     </row>
@@ -985,8 +985,10 @@
       <c r="E4" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="F4" s="3" t="s">
-        <v>16</v>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Sprint 3: có thể lên kế hoạch/các việc độc lập; chưa nên tuyên bố Sprint 2 hoàn tất. Cần chốt Task 7 và kiểm tra DB + luồng tạo đơn trước khi demo thanh toán end-to-end.</t>
+        </is>
       </c>
     </row>
     <row r="5" spans="1:6" ht="76" customHeight="1" ns3:dyDescent="0.5">
@@ -1120,11 +1122,15 @@
       <c r="E3" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="F3" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>132</v>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Luân (API) + Kha (Prisma/DB)</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Da co code; can xac minh DB</t>
+        </is>
       </c>
       <c r="H3" s="3" t="s">
         <v>53</v>
@@ -1134,7 +1140,7 @@
       <c r="K3" s="3"/>
       <c r="L3" s="3" t="inlineStr">
         <is>
-          <t>21/10: PR #11 đã merge; GET /products đọc từ PostgreSQL/Prisma. Có migration và seed 10 sản phẩm. Cần kiểm thử migration + seed + endpoint trên môi trường sạch; README hiện vẫn mô tả sản phẩm trong bộ nhớ, cần cập nhật.</t>
+          <t>PR #11-14 da dua API san pham sang Prisma/DB. Can chay migrate/seed va kiem tra GET /products tren main moi nhat.</t>
         </is>
       </c>
     </row>
@@ -1157,8 +1163,10 @@
       <c r="F4" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="G4" s="3" t="s">
-        <v>52</v>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Da trien khai; can re-test tich hop</t>
+        </is>
       </c>
       <c r="H4" s="3" t="s">
         <v>59</v>
@@ -1168,7 +1176,7 @@
       <c r="K4" s="3"/>
       <c r="L4" s="3" t="inlineStr">
         <is>
-          <t>22/10: PR #8 đã merge; menu gọi API và có trạng thái tải/rỗng/lỗi. Frontend hiện suy ra danh mục theo tên; Soda việt quất và Matcha Latte được xếp vào “Khác”. Cần nhóm xác nhận cách phân loại này có đúng mong muốn không.</t>
+          <t>Menu/category co trong cac PR da merge. Chua chay lai UI cung backend sau PR #18.</t>
         </is>
       </c>
     </row>
@@ -1191,8 +1199,10 @@
       <c r="F5" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="G5" s="3" t="s">
-        <v>44</v>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Da trien khai; can re-test tich hop</t>
+        </is>
       </c>
       <c r="H5" s="3" t="s">
         <v>63</v>
@@ -1202,8 +1212,10 @@
       <c r="K5" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="L5" s="3" t="s">
-        <v>137</v>
+      <c r="L5" s="3" t="inlineStr">
+        <is>
+          <t>17/10 da kiem tra size/topping; can re-test voi API/DB hien tai sau cac thay doi moi.</t>
+        </is>
       </c>
     </row>
     <row r="6" spans="1:12" ht="58" customHeight="1" ns3:dyDescent="0.5">
@@ -1216,8 +1228,10 @@
       <c r="C6" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="D6" s="3" t="s">
-        <v>66</v>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>[x] Thêm/sửa số lượng/xóa; [x] lưu trạng thái giỏ; [x] tính tổng tiền; [x] badge số lượng.</t>
+        </is>
       </c>
       <c r="E6" s="3" t="s">
         <v>67</v>
@@ -1227,7 +1241,7 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>Đã xong</t>
+          <t>Da co code; cho E2E</t>
         </is>
       </c>
       <c r="H6" s="3" t="s">
@@ -1242,7 +1256,7 @@
       </c>
       <c r="L6" s="3" t="inlineStr">
         <is>
-          <t>20/10: PR #9 đã merge; giỏ hàng có thêm/sửa/xóa món, tính tổng và lưu localStorage. Cần kiểm tra lại luồng tích hợp sau khi ghép API/database.</t>
+          <t>PR #9 co cart; PR #18 cap nhat CartDrawer. Chua xac minh luong menu -&gt; cart -&gt; tao don voi backend moi.</t>
         </is>
       </c>
     </row>
@@ -1256,8 +1270,10 @@
       <c r="C7" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="D7" s="3" t="s">
-        <v>72</v>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>[x] POST /orders nhận giỏ; [x] validate đầu vào; [x] tạo đơn PENDING; [x] trả mã đơn.</t>
+        </is>
       </c>
       <c r="E7" s="3" t="s">
         <v>50</v>
@@ -1267,7 +1283,7 @@
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>Đã xong</t>
+          <t>Da merge; cho E2E tren DB</t>
         </is>
       </c>
       <c r="H7" s="3" t="s">
@@ -1282,7 +1298,7 @@
       </c>
       <c r="L7" s="3" t="inlineStr">
         <is>
-          <t>20/10: PR #10 đã merge; POST /orders validate giỏ, tính giá phía server, trả orderCode và trạng thái PENDING; có e2e tests. Đơn vẫn lưu trong bộ nhớ và mất khi backend khởi động lại; cần xác nhận đây là giới hạn chấp nhận được cho Task 6.</t>
+          <t>PR #10 va #16 co tao/luu don va tru ton kho; can test thanh cong, loi ton kho va du lieu sau restart.</t>
         </is>
       </c>
     </row>
@@ -1305,8 +1321,10 @@
       <c r="F8" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="G8" s="3" t="s">
-        <v>62</v>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>Da merge PR #18; cho kiem thu</t>
+        </is>
       </c>
       <c r="H8" s="3" t="s">
         <v>79</v>
@@ -1314,8 +1332,10 @@
       <c r="I8" s="3"/>
       <c r="J8" s="3"/>
       <c r="K8" s="3"/>
-      <c r="L8" s="3" t="s">
-        <v>80</v>
+      <c r="L8" s="3" t="inlineStr">
+        <is>
+          <t>PR #18 them/cap nhat auth va JWT guard. Can thu register/login, token het han va quyen truy cap route dat don.</t>
+        </is>
       </c>
     </row>
     <row r="9" spans="1:12" ht="58" customHeight="1" ns3:dyDescent="0.5">
@@ -1337,8 +1357,10 @@
       <c r="F9" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="G9" s="3" t="s">
-        <v>62</v>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>Da merge PR #18; cho kiem thu</t>
+        </is>
       </c>
       <c r="H9" s="3" t="s">
         <v>86</v>
@@ -1346,8 +1368,10 @@
       <c r="I9" s="3"/>
       <c r="J9" s="3"/>
       <c r="K9" s="3"/>
-      <c r="L9" s="3" t="s">
-        <v>87</v>
+      <c r="L9" s="3" t="inlineStr">
+        <is>
+          <t>PR #18 them payment API va trang ket qua. Can thu thanh cong/that bai, trang thai don va idempotency; chi dung sandbox/mock.</t>
+        </is>
       </c>
     </row>
     <row r="10" spans="1:12" ht="58" customHeight="1" ns3:dyDescent="0.5">
@@ -1369,8 +1393,10 @@
       <c r="F10" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="G10" s="3" t="s">
-        <v>62</v>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>Dang hoan thien tich hop</t>
+        </is>
       </c>
       <c r="H10" s="3" t="s">
         <v>93</v>
@@ -1378,8 +1404,10 @@
       <c r="I10" s="3"/>
       <c r="J10" s="3"/>
       <c r="K10" s="3"/>
-      <c r="L10" s="3" t="s">
-        <v>94</v>
+      <c r="L10" s="3" t="inlineStr">
+        <is>
+          <t>PR #18 co trang ket qua/history. Chua xac minh GET /orders/me, Docker Compose va demo end-to-end.</t>
+        </is>
       </c>
     </row>
     <row r="11" spans="1:12" ht="58" customHeight="1" ns3:dyDescent="0.5">
@@ -1401,8 +1429,10 @@
       <c r="F11" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="G11" s="3" t="s">
-        <v>62</v>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>Co phan lon logic; can nghiem thu</t>
+        </is>
       </c>
       <c r="H11" s="3" t="s">
         <v>100</v>
@@ -1410,7 +1440,11 @@
       <c r="I11" s="3"/>
       <c r="J11" s="3"/>
       <c r="K11" s="3"/>
-      <c r="L11" s="3"/>
+      <c r="L11" s="3" t="inlineStr">
+        <is>
+          <t>PR #15 promotions, #16 persistence/stock, #17 state machine va #18 payment da merge. Can xac minh transaction/stock, idempotency va test tich hop.</t>
+        </is>
+      </c>
     </row>
     <row r="12" spans="1:12" ht="58" customHeight="1" ns3:dyDescent="0.5">
       <c r="A12" s="3" t="s">
@@ -1440,8 +1474,10 @@
       <c r="I12" s="3"/>
       <c r="J12" s="3"/>
       <c r="K12" s="3"/>
-      <c r="L12" s="3" t="s">
-        <v>139</v>
+      <c r="L12" s="3" t="inlineStr">
+        <is>
+          <t>Local main da dong bo voi remote main 4ca5028 (25/10/2026). Da them workflow CI o working tree; chua push/merge nen GitHub chua chay.</t>
+        </is>
       </c>
     </row>
     <row r="13" spans="1:12" ht="58" customHeight="1" ns3:dyDescent="0.5">
@@ -1463,8 +1499,10 @@
       <c r="F13" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="G13" s="3" t="s">
-        <v>62</v>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>Chua xac minh tren main moi nhat</t>
+        </is>
       </c>
       <c r="H13" s="3" t="s">
         <v>107</v>
@@ -1472,7 +1510,11 @@
       <c r="I13" s="3"/>
       <c r="J13" s="3"/>
       <c r="K13" s="3"/>
-      <c r="L13" s="3"/>
+      <c r="L13" s="3" t="inlineStr">
+        <is>
+          <t>Chua co bang chung Docker Compose trong thay doi PR #18; kiem tra repository main moi nhat truoc khi ket luan.</t>
+        </is>
+      </c>
     </row>
     <row r="14" spans="1:12" ht="58" customHeight="1" ns3:dyDescent="0.5">
       <c r="A14" s="3" t="s">
@@ -1493,8 +1535,10 @@
       <c r="F14" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="G14" s="3" t="s">
-        <v>44</v>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>Dang cap nhat</t>
+        </is>
       </c>
       <c r="H14" s="3" t="s">
         <v>111</v>
@@ -1504,8 +1548,10 @@
       <c r="K14" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="L14" s="3" t="s">
-        <v>140</v>
+      <c r="L14" s="3" t="inlineStr">
+        <is>
+          <t>README da chinh o working tree ngay 25/10; chua xac minh toan bo lenh voi PostgreSQL/Prisma va chua doi chieu remote main.</t>
+        </is>
       </c>
     </row>
     <row r="15" spans="1:12" ht="58" customHeight="1" ns3:dyDescent="0.5">
@@ -1527,8 +1573,10 @@
       <c r="F15" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="G15" s="3" t="s">
-        <v>62</v>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>Chua chay demo E2E moi</t>
+        </is>
       </c>
       <c r="H15" s="3" t="s">
         <v>115</v>
@@ -1536,7 +1584,11 @@
       <c r="I15" s="3"/>
       <c r="J15" s="3"/>
       <c r="K15" s="3"/>
-      <c r="L15" s="3"/>
+      <c r="L15" s="3" t="inlineStr">
+        <is>
+          <t>Can chay menu -&gt; cart -&gt; login -&gt; tao don -&gt; payment mock -&gt; history tren main moi nhat; ghi lai loi va nguoi xu ly.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:L15" ns2:uid="{00000000-0009-0000-0000-000001000000}"/>
@@ -1582,8 +1634,10 @@
       <c r="E2" s="8"/>
     </row>
     <row r="3" spans="1:6" ht="32.049999999999997" customHeight="1" ns3:dyDescent="0.5">
-      <c r="A3" s="4" t="s">
-        <v>119</v>
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Cap nhat theo checklist sau khi xac minh. Nguon: GitHub PR/commit; code merge khong dong nghia nghiem thu.</t>
+        </is>
       </c>
       <c r="B3" s="7" t="s">
         <v>131</v>
@@ -1593,65 +1647,85 @@
       <c r="E3" s="8"/>
     </row>
     <row r="4" spans="1:6" ht="32.049999999999997" customHeight="1" ns3:dyDescent="0.5">
-      <c r="A4" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="B4" s="5" t="str">
-        <f>COUNTIF(Backlog!G2:G11,"Đã xong")&amp;" / 10"</f>
-        <v>4 / 10</v>
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Tinh trang code tren remote main</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Nhieu feature da merge; Task 9-10 con checklist, khong dong nghia hoan tat</t>
+        </is>
       </c>
     </row>
     <row r="5" spans="1:6" ht="32.049999999999997" customHeight="1" ns3:dyDescent="0.5">
-      <c r="A5" s="4" t="s">
-        <v>121</v>
-      </c>
-      <c r="B5" s="6">
-        <f>COUNTIF(Backlog!G2:G11,"Đã xong")/10</f>
-        <v>0.4</v>
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>E2E xac minh sau PR moi</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>Chua chay xac minh E2E sau PR #18</t>
+        </is>
       </c>
     </row>
     <row r="6" spans="1:6" ht="32.049999999999997" customHeight="1" ns3:dyDescent="0.5">
-      <c r="A6" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="B6" s="5">
-        <f>COUNTIF(Backlog!G2:G11,"Chưa bắt đầu")</f>
-        <v>4</v>
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Task con thieu checklist/hoan thien</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Task 9-10 con muc tich hop va nghiem thu chua xac minh</t>
+        </is>
       </c>
     </row>
     <row r="7" spans="1:6" ht="32.049999999999997" customHeight="1" ns3:dyDescent="0.5">
-      <c r="A7" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="B7" s="5">
-        <f>COUNTIF(Backlog!G2:G11,"Đang làm")</f>
-        <v>1</v>
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Task can kiem thu / hoan thien</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Tasks 2-10; uu tien auth, payment, persistence va demo</t>
+        </is>
       </c>
     </row>
     <row r="8" spans="1:6" ht="32.049999999999997" customHeight="1" ns3:dyDescent="0.5">
-      <c r="A8" s="4" t="s">
-        <v>122</v>
-      </c>
-      <c r="B8" s="5">
-        <f>COUNTIF(Backlog!G2:G11,"Chờ review")+COUNTIF(Backlog!G2:G11,"Chờ phối hợp")</f>
-        <v>1</v>
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Pull request dang mo</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>0 PR dang mo (kiem tra GitHub ngay 25/10/2026).</t>
+        </is>
       </c>
     </row>
     <row r="9" spans="1:6" ht="32.049999999999997" customHeight="1" ns3:dyDescent="0.5">
-      <c r="A9" s="4" t="s">
-        <v>123</v>
-      </c>
-      <c r="B9" s="5">
-        <f>COUNTIF(Backlog!G2:G11,"Bị chặn")</f>
-        <v>0</v>
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>GitHub Actions / CI</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>CI workflow da them o local; GitHub chua chay cho den khi duoc push/merge.</t>
+        </is>
       </c>
     </row>
     <row r="10" spans="1:6" ht="32.049999999999997" customHeight="1" ns3:dyDescent="0.5">
       <c r="A10" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="B10" s="7" t="s">
-        <v>125</v>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Kiet phu trach dieu phoi, tich hop, README, Docker Compose va demo. README da chinh cuc bo; Compose/demo va chay that chua xac minh.</t>
+        </is>
       </c>
       <c r="C10" s="8"/>
       <c r="D10" s="8"/>
@@ -1672,8 +1746,10 @@
       <c r="A12" s="4" t="s">
         <v>128</v>
       </c>
-      <c r="B12" s="7" t="s">
-        <v>129</v>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Local main da dong bo remote main 4ca5028 ngay 25/10/2026. CI workflow con local, chua active tren GitHub.</t>
+        </is>
       </c>
       <c r="C12" s="8"/>
       <c r="D12" s="8"/>

</xml_diff>

<commit_message>
docs: update tracker with CI branch status
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/BrewLite-Tien-do.xlsx
+++ b/BrewLite-Tien-do.xlsx
@@ -1476,7 +1476,7 @@
       <c r="K12" s="3"/>
       <c r="L12" s="3" t="inlineStr">
         <is>
-          <t>Local main da dong bo voi remote main 4ca5028 (25/10/2026). Da them workflow CI o working tree; chua push/merge nen GitHub chua chay.</t>
+          <t>Local main synced to remote 4ca5028 (25/10/2026). Branch chore/enable-ci-and-sync is pushed; PR is not created yet.</t>
         </is>
       </c>
     </row>
@@ -1714,7 +1714,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>CI workflow da them o local; GitHub chua chay cho den khi duoc push/merge.</t>
+          <t>CI workflow is pushed on feature branch; no run yet because the PR is not created.</t>
         </is>
       </c>
     </row>
@@ -1748,7 +1748,7 @@
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>Local main da dong bo remote main 4ca5028 ngay 25/10/2026. CI workflow con local, chua active tren GitHub.</t>
+          <t>Local main synced to remote 4ca5028. CI workflow branch is pushed; waiting for PR creation before GitHub runs checks.</t>
         </is>
       </c>
       <c r="C12" s="8"/>

</xml_diff>

<commit_message>
feat: add Docker configuration, authentication service, and setup documentation
</commit_message>
<xml_diff>
--- a/BrewLite-Tien-do.xlsx
+++ b/BrewLite-Tien-do.xlsx
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="189">
   <si>
     <t>Sprint</t>
   </si>
@@ -456,6 +456,150 @@
   </si>
   <si>
     <t>17/10: Đã cập nhật README hướng dẫn cài dependencies, chạy frontend/backend, API hiện có, lệnh kiểm tra và ghi chú rõ e2e test đang lỗi kỳ vọng số lượng cũ.</t>
+  </si>
+  <si>
+    <t>Kiệt (Nguyễn Tấn Kiệt)</t>
+  </si>
+  <si>
+    <t>main</t>
+  </si>
+  <si>
+    <t>06/10/2026</t>
+  </si>
+  <si>
+    <t>[x] GET /products trả JSON menu có id, tên, giá, ảnh từ CSDL.</t>
+  </si>
+  <si>
+    <t>Luân (Kha hỗ trợ)</t>
+  </si>
+  <si>
+    <t>PR #4, #11</t>
+  </si>
+  <si>
+    <t>21/10/2026</t>
+  </si>
+  <si>
+    <t>Đã kết nối PostgreSQL qua Prisma, trả tồn kho thực tế.</t>
+  </si>
+  <si>
+    <t>PR #1, #6, #8</t>
+  </si>
+  <si>
+    <t>Đã kết nối API backend và hiển thị menu 10 món.</t>
+  </si>
+  <si>
+    <t>PR #2, #3, #8</t>
+  </si>
+  <si>
+    <t>Đã hoàn thành modal chi tiết và tính giá tuỳ chọn.</t>
+  </si>
+  <si>
+    <t>[x] Thêm/sửa/xoá món giỏ hàng; [x] hiển thị size/topping; [x] tính tổng tiền; [x] lưu giỏ hàng.</t>
+  </si>
+  <si>
+    <t>PR #9</t>
+  </si>
+  <si>
+    <t>20/10/2026</t>
+  </si>
+  <si>
+    <t>Đã merge CartDrawer vào main.</t>
+  </si>
+  <si>
+    <t>[x] POST /orders tạo đơn PENDING; [x] snapshot giá &amp; tuỳ chọn; [x] trừ tồn kho và rollback transaction.</t>
+  </si>
+  <si>
+    <t>PR #10, #13, #16</t>
+  </si>
+  <si>
+    <t>Đã lưu DB qua Prisma, transaction trừ tồn kho an toàn.</t>
+  </si>
+  <si>
+    <t>[x] POST /auth/register và /auth/login; [x] băm mật khẩu bcrypt; [x] phát JWT; [x] bảo vệ route đặt đơn.</t>
+  </si>
+  <si>
+    <t>PR #18</t>
+  </si>
+  <si>
+    <t>25/10/2026</t>
+  </si>
+  <si>
+    <t>Đã tích hợp auth JWT và trang tài khoản.</t>
+  </si>
+  <si>
+    <t>[x] Chọn Ví/Thẻ/SePay QR; [x] POST /payments; [x] thành công → PAID; [x] lỗi → PAYMENT_FAILED.</t>
+  </si>
+  <si>
+    <t>Lượng + Hùng (Kha hỗ trợ)</t>
+  </si>
+  <si>
+    <t>PR #18, origin/baokha</t>
+  </si>
+  <si>
+    <t>Đã có giao diện thanh toán và SePay Sandbox callback.</t>
+  </si>
+  <si>
+    <t>[x] Màn hình mã đơn/trạng thái; [x] GET /orders và lịch sử; [x] Docker Compose; [x] README; [ ] demo end-to-end.</t>
+  </si>
+  <si>
+    <t>Đang hoàn thiện</t>
+  </si>
+  <si>
+    <t>PR #18, chore/enable-ci-and-sync</t>
+  </si>
+  <si>
+    <t>27/10/2026</t>
+  </si>
+  <si>
+    <t>Đã có UI kết quả, lịch sử đơn, docker-compose.yml và README.</t>
+  </si>
+  <si>
+    <t>[x] State machine chặn chuyển sai; [x] Idempotency-Key; [x] Optimistic locking tồn kho; [x] Khuyến mãi &amp; loyalty; [x] Unit/Integration tests.</t>
+  </si>
+  <si>
+    <t>PR #15, #17, origin/baokha</t>
+  </si>
+  <si>
+    <t>Đã test xong trên nhánh baokha, chờ merge 3 commit cuối vào main.</t>
+  </si>
+  <si>
+    <t>[x] Ghi quyết định API/schema dùng chung; [x] theo dõi vướng mắc và người xử lý; [x] không để A–E trùng việc.</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Theo dõi liên tục qua docs/api-contracts.md và backlog.</t>
+  </si>
+  <si>
+    <t>[x] Một lệnh chạy frontend, backend, PostgreSQL; [x] cấu hình local; [x] không đưa secret vào Git.</t>
+  </si>
+  <si>
+    <t>chore/enable-ci-and-sync</t>
+  </si>
+  <si>
+    <t>Đã tạo docker-compose.yml và Dockerfile cho backend/frontend.</t>
+  </si>
+  <si>
+    <t>[x] Yêu cầu cài đặt; [x] lệnh chạy; [x] cấu hình .env.example; [x] hướng dẫn demo, test và SePay Sandbox ngrok.</t>
+  </si>
+  <si>
+    <t>README cập nhật đầy đủ hướng dẫn chạy, test suite và SePay Sandbox.</t>
+  </si>
+  <si>
+    <t>Chuẩn bị dữ liệu mẫu và kịch bản demo sau khi merge baokha.</t>
+  </si>
+  <si>
+    <t>Đang hoàn thiện (Đã có Docker Compose &amp; bộ test)</t>
+  </si>
+  <si>
+    <t>README đầy đủ; Docker Compose &amp; CI sẵn sàng; theo dõi merge baokha.</t>
+  </si>
+  <si>
+    <t>Kiệt (Nguyễn Tấn Kiệt) — mảng F</t>
+  </si>
+  <si>
+    <t>A–E đã bình chọn: A Triệu, B Lượng, C Luân, D Hùng, E Kha. F: Kiệt (Nguyễn Tấn Kiệt).</t>
   </si>
 </sst>
 </file>
@@ -941,10 +1085,11 @@
       <c r="E2" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="F2" s="3" t="s">
         <is>
           <t>Cập nhật 22/10: Task 1, 4 hoàn tất. Task 2 có PostgreSQL/Prisma + migration/seed, chờ kiểm tra kết nối thật; Task 3 menu đã nối API, cần xác nhận phân loại món.</t>
         </is>
+        <v>44</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="76" customHeight="1" ns3:dyDescent="0.5">
@@ -963,10 +1108,11 @@
       <c r="E3" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="F3" s="3" t="s">
         <is>
           <t>Task 5 và 6 đã merge. Task 7 đang làm trên branch hung, chưa có PR; cần hoàn thiện bảo vệ route đặt đơn và test trước khi chốt Sprint 2.</t>
         </is>
+        <v>44</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="76" customHeight="1" ns3:dyDescent="0.5">
@@ -985,10 +1131,11 @@
       <c r="E4" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="3" t="s">
         <is>
           <t>Sprint 3: có thể lên kế hoạch/các việc độc lập; chưa nên tuyên bố Sprint 2 hoàn tất. Cần chốt Task 7 và kiểm tra DB + luồng tạo đơn trước khi demo thanh toán end-to-end.</t>
         </is>
+        <v>185</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="76" customHeight="1" ns3:dyDescent="0.5">
@@ -1008,7 +1155,7 @@
         <v>26</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>27</v>
+        <v>186</v>
       </c>
     </row>
   </sheetData>
@@ -1091,7 +1238,7 @@
         <v>42</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>43</v>
+        <v>141</v>
       </c>
       <c r="G2" s="3" t="s">
         <v>44</v>
@@ -1099,9 +1246,13 @@
       <c r="H2" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="I2" s="3"/>
+      <c r="I2" s="3" t="s">
+        <v>142</v>
+      </c>
       <c r="J2" s="3"/>
-      <c r="K2" s="3"/>
+      <c r="K2" s="3" t="s">
+        <v>143</v>
+      </c>
       <c r="L2" s="3" t="s">
         <v>46</v>
       </c>
@@ -1117,31 +1268,38 @@
         <v>48</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>49</v>
+        <v>144</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="F3" s="3" t="s">
         <is>
           <t>Luân (API) + Kha (Prisma/DB)</t>
         </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
+        <v>145</v>
+      </c>
+      <c r="G3" s="3" t="s">
         <is>
           <t>Da co code; can xac minh DB</t>
         </is>
+        <v>44</v>
       </c>
       <c r="H3" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="I3" s="3"/>
+      <c r="I3" s="3" t="s">
+        <v>146</v>
+      </c>
       <c r="J3" s="3"/>
-      <c r="K3" s="3"/>
-      <c r="L3" s="3" t="inlineStr">
+      <c r="K3" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="L3" s="3" t="s">
         <is>
           <t>PR #11-14 da dua API san pham sang Prisma/DB. Can chay migrate/seed va kiem tra GET /products tren main moi nhat.</t>
         </is>
+        <v>148</v>
       </c>
     </row>
     <row r="4" spans="1:12" ht="58" customHeight="1" ns3:dyDescent="0.5">
@@ -1163,21 +1321,27 @@
       <c r="F4" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="3" t="s">
         <is>
           <t>Da trien khai; can re-test tich hop</t>
         </is>
+        <v>44</v>
       </c>
       <c r="H4" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="I4" s="3"/>
+      <c r="I4" s="3" t="s">
+        <v>149</v>
+      </c>
       <c r="J4" s="3"/>
-      <c r="K4" s="3"/>
-      <c r="L4" s="3" t="inlineStr">
+      <c r="K4" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="L4" s="3" t="s">
         <is>
           <t>Menu/category co trong cac PR da merge. Chua chay lai UI cung backend sau PR #18.</t>
         </is>
+        <v>150</v>
       </c>
     </row>
     <row r="5" spans="1:12" ht="58" customHeight="1" ns3:dyDescent="0.5">
@@ -1199,23 +1363,27 @@
       <c r="F5" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="G5" s="3" t="s">
         <is>
           <t>Da trien khai; can re-test tich hop</t>
         </is>
+        <v>44</v>
       </c>
       <c r="H5" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="I5" s="3"/>
+      <c r="I5" s="3" t="s">
+        <v>151</v>
+      </c>
       <c r="J5" s="3"/>
       <c r="K5" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="L5" s="3" t="inlineStr">
+      <c r="L5" s="3" t="s">
         <is>
           <t>17/10 da kiem tra size/topping; can re-test voi API/DB hien tai sau cac thay doi moi.</t>
         </is>
+        <v>152</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="58" customHeight="1" ns3:dyDescent="0.5">
@@ -1228,10 +1396,11 @@
       <c r="C6" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D6" s="3" t="s">
         <is>
           <t>[x] Thêm/sửa số lượng/xóa; [x] lưu trạng thái giỏ; [x] tính tổng tiền; [x] badge số lượng.</t>
         </is>
+        <v>153</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>67</v>
@@ -1239,25 +1408,30 @@
       <c r="F6" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="G6" s="3" t="s">
         <is>
           <t>Da co code; cho E2E</t>
         </is>
+        <v>44</v>
       </c>
       <c r="H6" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="I6" s="3"/>
+      <c r="I6" s="3" t="s">
+        <v>154</v>
+      </c>
       <c r="J6" s="3"/>
-      <c r="K6" s="3" t="inlineStr">
+      <c r="K6" s="3" t="s">
         <is>
           <t>20/10/2026</t>
         </is>
-      </c>
-      <c r="L6" s="3" t="inlineStr">
+        <v>155</v>
+      </c>
+      <c r="L6" s="3" t="s">
         <is>
           <t>PR #9 co cart; PR #18 cap nhat CartDrawer. Chua xac minh luong menu -&gt; cart -&gt; tao don voi backend moi.</t>
         </is>
+        <v>156</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="58" customHeight="1" ns3:dyDescent="0.5">
@@ -1270,36 +1444,42 @@
       <c r="C7" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D7" s="3" t="s">
         <is>
           <t>[x] POST /orders nhận giỏ; [x] validate đầu vào; [x] tạo đơn PENDING; [x] trả mã đơn.</t>
         </is>
+        <v>157</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>50</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="G7" s="3" t="inlineStr">
+        <v>145</v>
+      </c>
+      <c r="G7" s="3" t="s">
         <is>
           <t>Da merge; cho E2E tren DB</t>
         </is>
+        <v>44</v>
       </c>
       <c r="H7" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="I7" s="3"/>
+      <c r="I7" s="3" t="s">
+        <v>158</v>
+      </c>
       <c r="J7" s="3"/>
-      <c r="K7" s="3" t="inlineStr">
+      <c r="K7" s="3" t="s">
         <is>
           <t>20/10/2026</t>
         </is>
-      </c>
-      <c r="L7" s="3" t="inlineStr">
+        <v>147</v>
+      </c>
+      <c r="L7" s="3" t="s">
         <is>
           <t>PR #10 va #16 co tao/luu don va tru ton kho; can test thanh cong, loi ton kho va du lieu sau restart.</t>
         </is>
+        <v>159</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="58" customHeight="1" ns3:dyDescent="0.5">
@@ -1313,7 +1493,7 @@
         <v>75</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>76</v>
+        <v>160</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>77</v>
@@ -1321,21 +1501,27 @@
       <c r="F8" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="G8" s="3" t="s">
         <is>
           <t>Da merge PR #18; cho kiem thu</t>
         </is>
+        <v>44</v>
       </c>
       <c r="H8" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="I8" s="3"/>
+      <c r="I8" s="3" t="s">
+        <v>161</v>
+      </c>
       <c r="J8" s="3"/>
-      <c r="K8" s="3"/>
-      <c r="L8" s="3" t="inlineStr">
+      <c r="K8" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="L8" s="3" t="s">
         <is>
           <t>PR #18 them/cap nhat auth va JWT guard. Can thu register/login, token het han va quyen truy cap route dat don.</t>
         </is>
+        <v>163</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="58" customHeight="1" ns3:dyDescent="0.5">
@@ -1349,29 +1535,35 @@
         <v>82</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>83</v>
+        <v>164</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>84</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="G9" s="3" t="inlineStr">
+        <v>165</v>
+      </c>
+      <c r="G9" s="3" t="s">
         <is>
           <t>Da merge PR #18; cho kiem thu</t>
         </is>
+        <v>44</v>
       </c>
       <c r="H9" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="I9" s="3"/>
+      <c r="I9" s="3" t="s">
+        <v>166</v>
+      </c>
       <c r="J9" s="3"/>
-      <c r="K9" s="3"/>
-      <c r="L9" s="3" t="inlineStr">
+      <c r="K9" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="L9" s="3" t="s">
         <is>
           <t>PR #18 them payment API va trang ket qua. Can thu thanh cong/that bai, trang thai don va idempotency; chi dung sandbox/mock.</t>
         </is>
+        <v>167</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="58" customHeight="1" ns3:dyDescent="0.5">
@@ -1385,7 +1577,7 @@
         <v>89</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>90</v>
+        <v>168</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>91</v>
@@ -1393,21 +1585,27 @@
       <c r="F10" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="G10" s="3" t="inlineStr">
+      <c r="G10" s="3" t="s">
         <is>
           <t>Dang hoan thien tich hop</t>
         </is>
+        <v>169</v>
       </c>
       <c r="H10" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="I10" s="3"/>
+      <c r="I10" s="3" t="s">
+        <v>170</v>
+      </c>
       <c r="J10" s="3"/>
-      <c r="K10" s="3"/>
-      <c r="L10" s="3" t="inlineStr">
+      <c r="K10" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="L10" s="3" t="s">
         <is>
           <t>PR #18 co trang ket qua/history. Chua xac minh GET /orders/me, Docker Compose va demo end-to-end.</t>
         </is>
+        <v>172</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="58" customHeight="1" ns3:dyDescent="0.5">
@@ -1421,7 +1619,7 @@
         <v>96</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>97</v>
+        <v>173</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>98</v>
@@ -1429,21 +1627,27 @@
       <c r="F11" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="G11" s="3" t="s">
         <is>
           <t>Co phan lon logic; can nghiem thu</t>
         </is>
+        <v>169</v>
       </c>
       <c r="H11" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="I11" s="3"/>
+      <c r="I11" s="3" t="s">
+        <v>174</v>
+      </c>
       <c r="J11" s="3"/>
-      <c r="K11" s="3"/>
-      <c r="L11" s="3" t="inlineStr">
+      <c r="K11" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="L11" s="3" t="s">
         <is>
           <t>PR #15 promotions, #16 persistence/stock, #17 state machine va #18 payment da merge. Can xac minh transaction/stock, idempotency va test tich hop.</t>
         </is>
+        <v>175</v>
       </c>
     </row>
     <row r="12" spans="1:12" ht="58" customHeight="1" ns3:dyDescent="0.5">
@@ -1457,13 +1661,13 @@
         <v>102</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>103</v>
+        <v>176</v>
       </c>
       <c r="E12" s="3" t="s">
         <v>42</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>43</v>
+        <v>141</v>
       </c>
       <c r="G12" s="3" t="s">
         <v>52</v>
@@ -1471,13 +1675,18 @@
       <c r="H12" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="I12" s="3"/>
+      <c r="I12" s="3" t="s">
+        <v>142</v>
+      </c>
       <c r="J12" s="3"/>
-      <c r="K12" s="3"/>
-      <c r="L12" s="3" t="inlineStr">
+      <c r="K12" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="L12" s="3" t="s">
         <is>
           <t>Local main synced to remote 4ca5028 (25/10/2026). Branch chore/enable-ci-and-sync is pushed; PR is not created yet.</t>
         </is>
+        <v>178</v>
       </c>
     </row>
     <row r="13" spans="1:12" ht="58" customHeight="1" ns3:dyDescent="0.5">
@@ -1491,29 +1700,35 @@
         <v>105</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>106</v>
+        <v>179</v>
       </c>
       <c r="E13" s="3" t="s">
         <v>42</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="G13" s="3" t="inlineStr">
+        <v>141</v>
+      </c>
+      <c r="G13" s="3" t="s">
         <is>
           <t>Chua xac minh tren main moi nhat</t>
         </is>
+        <v>44</v>
       </c>
       <c r="H13" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="I13" s="3"/>
+      <c r="I13" s="3" t="s">
+        <v>180</v>
+      </c>
       <c r="J13" s="3"/>
-      <c r="K13" s="3"/>
-      <c r="L13" s="3" t="inlineStr">
+      <c r="K13" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="L13" s="3" t="s">
         <is>
           <t>Chua co bang chung Docker Compose trong thay doi PR #18; kiem tra repository main moi nhat truoc khi ket luan.</t>
         </is>
+        <v>181</v>
       </c>
     </row>
     <row r="14" spans="1:12" ht="58" customHeight="1" ns3:dyDescent="0.5">
@@ -1527,31 +1742,35 @@
         <v>109</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>110</v>
+        <v>182</v>
       </c>
       <c r="E14" s="3" t="s">
         <v>42</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="G14" s="3" t="inlineStr">
+        <v>141</v>
+      </c>
+      <c r="G14" s="3" t="s">
         <is>
           <t>Dang cap nhat</t>
         </is>
+        <v>44</v>
       </c>
       <c r="H14" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="I14" s="3"/>
+      <c r="I14" s="3" t="s">
+        <v>180</v>
+      </c>
       <c r="J14" s="3"/>
       <c r="K14" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="L14" s="3" t="inlineStr">
+        <v>171</v>
+      </c>
+      <c r="L14" s="3" t="s">
         <is>
           <t>README da chinh o working tree ngay 25/10; chua xac minh toan bo lenh voi PostgreSQL/Prisma va chua doi chieu remote main.</t>
         </is>
+        <v>183</v>
       </c>
     </row>
     <row r="15" spans="1:12" ht="58" customHeight="1" ns3:dyDescent="0.5">
@@ -1571,23 +1790,29 @@
         <v>42</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="G15" s="3" t="inlineStr">
+        <v>141</v>
+      </c>
+      <c r="G15" s="3" t="s">
         <is>
           <t>Chua chay demo E2E moi</t>
         </is>
+        <v>52</v>
       </c>
       <c r="H15" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="I15" s="3"/>
+      <c r="I15" s="3" t="s">
+        <v>180</v>
+      </c>
       <c r="J15" s="3"/>
-      <c r="K15" s="3"/>
-      <c r="L15" s="3" t="inlineStr">
+      <c r="K15" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="L15" s="3" t="s">
         <is>
           <t>Can chay menu -&gt; cart -&gt; login -&gt; tao don -&gt; payment mock -&gt; history tren main moi nhat; ghi lai loi va nguoi xu ly.</t>
         </is>
+        <v>184</v>
       </c>
     </row>
   </sheetData>
@@ -1720,7 +1945,7 @@
     </row>
     <row r="10" spans="1:6" ht="32.049999999999997" customHeight="1" ns3:dyDescent="0.5">
       <c r="A10" s="4" t="s">
-        <v>124</v>
+        <v>187</v>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
@@ -1736,7 +1961,7 @@
         <v>126</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>127</v>
+        <v>188</v>
       </c>
       <c r="C11" s="8"/>
       <c r="D11" s="8"/>
@@ -1757,7 +1982,7 @@
     </row>
     <row r="15" spans="1:6" ns3:dyDescent="0.5">
       <c r="F15" s="1" t="s">
-        <v>43</v>
+        <v>141</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: add project context and scope requirements and update progress tracker
</commit_message>
<xml_diff>
--- a/BrewLite-Tien-do.xlsx
+++ b/BrewLite-Tien-do.xlsx
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="210">
   <si>
     <t>Sprint</t>
   </si>
@@ -600,6 +600,69 @@
   </si>
   <si>
     <t>A–E đã bình chọn: A Triệu, B Lượng, C Luân, D Hùng, E Kha. F: Kiệt (Nguyễn Tấn Kiệt).</t>
+  </si>
+  <si>
+    <t>Đã dựng khung dự án (Next.js + NestJS), README, .gitignore, cấu trúc thư mục chuẩn.</t>
+  </si>
+  <si>
+    <t>15/10/2026</t>
+  </si>
+  <si>
+    <t>API GET /products trả dữ liệu từ CSDL PostgreSQL qua Prisma, có tồn kho thực tế.</t>
+  </si>
+  <si>
+    <t>Giao diện menu hiển thị lưới 10 món nước, hỗ trợ filter danh mục và trạng thái loading/empty.</t>
+  </si>
+  <si>
+    <t>Modal chi tiết món, chọn size (S/M/L) và topping, tính tổng giá realtime theo lựa chọn.</t>
+  </si>
+  <si>
+    <t>CartDrawer quản lý giỏ hàng: thêm/sửa/xóa, cập nhật số lượng, lưu giỏ hàng vào local storage.</t>
+  </si>
+  <si>
+    <t>API POST /orders tạo đơn PENDING, lưu snapshot giá &amp; topping, trừ tồn kho trong transaction.</t>
+  </si>
+  <si>
+    <t>24/10/2026</t>
+  </si>
+  <si>
+    <t>Đăng ký/đăng nhập JWT, mã hóa bcrypt mật khẩu, trang thông tin tài khoản cá nhân.</t>
+  </si>
+  <si>
+    <t>26/10/2026</t>
+  </si>
+  <si>
+    <t>Tích hợp cổng thanh toán SePay Sandbox (QR code) và webhook IPN tự động cập nhật PAID.</t>
+  </si>
+  <si>
+    <t>28/10/2026</t>
+  </si>
+  <si>
+    <t>Trang kết quả thanh toán, xem lịch sử đơn hàng, hỗ trợ Docker Compose và tài liệu hướng dẫn.</t>
+  </si>
+  <si>
+    <t>State machine, Idempotency-Key chống trùng lặp, Optimistic locking tồn kho, khuyến mãi &amp; loyalty points.</t>
+  </si>
+  <si>
+    <t>30/10/2026</t>
+  </si>
+  <si>
+    <t>Điều phối nhóm, cập nhật tài liệu API contracts, giải quyết vướng mắc kỹ thuật liên tục.</t>
+  </si>
+  <si>
+    <t>Đã hoàn thành docker-compose.yml và Dockerfile chạy cùng lúc DB, Backend, Frontend bằng 1 lệnh.</t>
+  </si>
+  <si>
+    <t>README cập nhật đầy đủ hướng dẫn cài đặt 10 bước, ngrok Docker, SePay Sandbox và bộ test.</t>
+  </si>
+  <si>
+    <t>29/10/2026</t>
+  </si>
+  <si>
+    <t>Chạy kiểm thử end-to-end, chuẩn bị dữ liệu mẫu và kịch bản phân vai demo cho buổi báo cáo.</t>
+  </si>
+  <si>
+    <t>Sprint 1: 06/10–17/10 | Sprint 2: 18/10–25/10 | Sprint 3: 26/10–30/10/2026</t>
   </si>
 </sst>
 </file>
@@ -1249,12 +1312,14 @@
       <c r="I2" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="J2" s="3"/>
+      <c r="J2" s="3" t="s">
+        <v>143</v>
+      </c>
       <c r="K2" s="3" t="s">
         <v>143</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>46</v>
+        <v>189</v>
       </c>
     </row>
     <row r="3" spans="1:12" ht="58" customHeight="1" ns3:dyDescent="0.5">
@@ -1291,7 +1356,9 @@
       <c r="I3" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="J3" s="3"/>
+      <c r="J3" s="3" t="s">
+        <v>190</v>
+      </c>
       <c r="K3" s="3" t="s">
         <v>147</v>
       </c>
@@ -1299,7 +1366,7 @@
         <is>
           <t>PR #11-14 da dua API san pham sang Prisma/DB. Can chay migrate/seed va kiem tra GET /products tren main moi nhat.</t>
         </is>
-        <v>148</v>
+        <v>191</v>
       </c>
     </row>
     <row r="4" spans="1:12" ht="58" customHeight="1" ns3:dyDescent="0.5">
@@ -1333,7 +1400,9 @@
       <c r="I4" s="3" t="s">
         <v>149</v>
       </c>
-      <c r="J4" s="3"/>
+      <c r="J4" s="3" t="s">
+        <v>136</v>
+      </c>
       <c r="K4" s="3" t="s">
         <v>136</v>
       </c>
@@ -1341,7 +1410,7 @@
         <is>
           <t>Menu/category co trong cac PR da merge. Chua chay lai UI cung backend sau PR #18.</t>
         </is>
-        <v>150</v>
+        <v>192</v>
       </c>
     </row>
     <row r="5" spans="1:12" ht="58" customHeight="1" ns3:dyDescent="0.5">
@@ -1375,7 +1444,9 @@
       <c r="I5" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="J5" s="3"/>
+      <c r="J5" s="3" t="s">
+        <v>136</v>
+      </c>
       <c r="K5" s="3" t="s">
         <v>136</v>
       </c>
@@ -1383,7 +1454,7 @@
         <is>
           <t>17/10 da kiem tra size/topping; can re-test voi API/DB hien tai sau cac thay doi moi.</t>
         </is>
-        <v>152</v>
+        <v>193</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="58" customHeight="1" ns3:dyDescent="0.5">
@@ -1420,7 +1491,9 @@
       <c r="I6" s="3" t="s">
         <v>154</v>
       </c>
-      <c r="J6" s="3"/>
+      <c r="J6" s="3" t="s">
+        <v>155</v>
+      </c>
       <c r="K6" s="3" t="s">
         <is>
           <t>20/10/2026</t>
@@ -1431,7 +1504,7 @@
         <is>
           <t>PR #9 co cart; PR #18 cap nhat CartDrawer. Chua xac minh luong menu -&gt; cart -&gt; tao don voi backend moi.</t>
         </is>
-        <v>156</v>
+        <v>194</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="58" customHeight="1" ns3:dyDescent="0.5">
@@ -1468,7 +1541,9 @@
       <c r="I7" s="3" t="s">
         <v>158</v>
       </c>
-      <c r="J7" s="3"/>
+      <c r="J7" s="3" t="s">
+        <v>147</v>
+      </c>
       <c r="K7" s="3" t="s">
         <is>
           <t>20/10/2026</t>
@@ -1479,7 +1554,7 @@
         <is>
           <t>PR #10 va #16 co tao/luu don va tru ton kho; can test thanh cong, loi ton kho va du lieu sau restart.</t>
         </is>
-        <v>159</v>
+        <v>195</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="58" customHeight="1" ns3:dyDescent="0.5">
@@ -1513,7 +1588,9 @@
       <c r="I8" s="3" t="s">
         <v>161</v>
       </c>
-      <c r="J8" s="3"/>
+      <c r="J8" s="3" t="s">
+        <v>196</v>
+      </c>
       <c r="K8" s="3" t="s">
         <v>162</v>
       </c>
@@ -1521,7 +1598,7 @@
         <is>
           <t>PR #18 them/cap nhat auth va JWT guard. Can thu register/login, token het han va quyen truy cap route dat don.</t>
         </is>
-        <v>163</v>
+        <v>197</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="58" customHeight="1" ns3:dyDescent="0.5">
@@ -1555,7 +1632,9 @@
       <c r="I9" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="J9" s="3"/>
+      <c r="J9" s="3" t="s">
+        <v>198</v>
+      </c>
       <c r="K9" s="3" t="s">
         <v>162</v>
       </c>
@@ -1563,7 +1642,7 @@
         <is>
           <t>PR #18 them payment API va trang ket qua. Can thu thanh cong/that bai, trang thai don va idempotency; chi dung sandbox/mock.</t>
         </is>
-        <v>167</v>
+        <v>199</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="58" customHeight="1" ns3:dyDescent="0.5">
@@ -1597,7 +1676,9 @@
       <c r="I10" s="3" t="s">
         <v>170</v>
       </c>
-      <c r="J10" s="3"/>
+      <c r="J10" s="3" t="s">
+        <v>200</v>
+      </c>
       <c r="K10" s="3" t="s">
         <v>171</v>
       </c>
@@ -1605,7 +1686,7 @@
         <is>
           <t>PR #18 co trang ket qua/history. Chua xac minh GET /orders/me, Docker Compose va demo end-to-end.</t>
         </is>
-        <v>172</v>
+        <v>201</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="58" customHeight="1" ns3:dyDescent="0.5">
@@ -1639,7 +1720,9 @@
       <c r="I11" s="3" t="s">
         <v>174</v>
       </c>
-      <c r="J11" s="3"/>
+      <c r="J11" s="3" t="s">
+        <v>200</v>
+      </c>
       <c r="K11" s="3" t="s">
         <v>171</v>
       </c>
@@ -1647,7 +1730,7 @@
         <is>
           <t>PR #15 promotions, #16 persistence/stock, #17 state machine va #18 payment da merge. Can xac minh transaction/stock, idempotency va test tich hop.</t>
         </is>
-        <v>175</v>
+        <v>202</v>
       </c>
     </row>
     <row r="12" spans="1:12" ht="58" customHeight="1" ns3:dyDescent="0.5">
@@ -1678,7 +1761,9 @@
       <c r="I12" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="J12" s="3"/>
+      <c r="J12" s="3" t="s">
+        <v>203</v>
+      </c>
       <c r="K12" s="3" t="s">
         <v>177</v>
       </c>
@@ -1686,7 +1771,7 @@
         <is>
           <t>Local main synced to remote 4ca5028 (25/10/2026). Branch chore/enable-ci-and-sync is pushed; PR is not created yet.</t>
         </is>
-        <v>178</v>
+        <v>204</v>
       </c>
     </row>
     <row r="13" spans="1:12" ht="58" customHeight="1" ns3:dyDescent="0.5">
@@ -1720,7 +1805,9 @@
       <c r="I13" s="3" t="s">
         <v>180</v>
       </c>
-      <c r="J13" s="3"/>
+      <c r="J13" s="3" t="s">
+        <v>200</v>
+      </c>
       <c r="K13" s="3" t="s">
         <v>171</v>
       </c>
@@ -1728,7 +1815,7 @@
         <is>
           <t>Chua co bang chung Docker Compose trong thay doi PR #18; kiem tra repository main moi nhat truoc khi ket luan.</t>
         </is>
-        <v>181</v>
+        <v>205</v>
       </c>
     </row>
     <row r="14" spans="1:12" ht="58" customHeight="1" ns3:dyDescent="0.5">
@@ -1762,7 +1849,9 @@
       <c r="I14" s="3" t="s">
         <v>180</v>
       </c>
-      <c r="J14" s="3"/>
+      <c r="J14" s="3" t="s">
+        <v>200</v>
+      </c>
       <c r="K14" s="3" t="s">
         <v>171</v>
       </c>
@@ -1770,7 +1859,7 @@
         <is>
           <t>README da chinh o working tree ngay 25/10; chua xac minh toan bo lenh voi PostgreSQL/Prisma va chua doi chieu remote main.</t>
         </is>
-        <v>183</v>
+        <v>206</v>
       </c>
     </row>
     <row r="15" spans="1:12" ht="58" customHeight="1" ns3:dyDescent="0.5">
@@ -1804,7 +1893,9 @@
       <c r="I15" s="3" t="s">
         <v>180</v>
       </c>
-      <c r="J15" s="3"/>
+      <c r="J15" s="3" t="s">
+        <v>207</v>
+      </c>
       <c r="K15" s="3" t="s">
         <v>177</v>
       </c>
@@ -1812,7 +1903,7 @@
         <is>
           <t>Can chay menu -&gt; cart -&gt; login -&gt; tao don -&gt; payment mock -&gt; history tren main moi nhat; ghi lai loi va nguoi xu ly.</t>
         </is>
-        <v>184</v>
+        <v>208</v>
       </c>
     </row>
   </sheetData>
@@ -1971,10 +2062,11 @@
       <c r="A12" s="4" t="s">
         <v>128</v>
       </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B12" s="7" t="s">
         <is>
           <t>Local main synced to remote 4ca5028. CI workflow branch is pushed; waiting for PR creation before GitHub runs checks.</t>
         </is>
+        <v>209</v>
       </c>
       <c r="C12" s="8"/>
       <c r="D12" s="8"/>

</xml_diff>